<commit_message>
fix: update ePO 5 package CMs for fixes on XPath conditions
</commit_message>
<xml_diff>
--- a/mappings/package_eforms_sdk1.3_epo5.2/transformation/conceptual_mappings.xlsx
+++ b/mappings/package_eforms_sdk1.3_epo5.2/transformation/conceptual_mappings.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14465" uniqueCount="5502">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14465" uniqueCount="5503">
   <si>
     <t>Field</t>
   </si>
@@ -2885,7 +2885,7 @@
     <t>/*/cac:ProcurementProjectLot[cbc:ID/@schemeName='Lot']/cac:TenderingProcess/cac:ContractingSystem/cbc:ContractingSystemTypeCode[@listName='dps-usage']</t>
   </si>
   <si>
-    <t>not(cbc:ContractingSystemTypeCode/text()='none')</t>
+    <t>not(cac:ContractingSystem/cbc:ContractingSystemTypeCode/text()='none')</t>
   </si>
   <si>
     <t>epo:Lot / epo:DynamicPurchaseSystemTechnique / at-voc:dps-usage</t>
@@ -15335,6 +15335,9 @@
   </si>
   <si>
     <t>/*/cac:ProcurementProjectLot[cbc:ID/@schemeName='Part']/cac:TenderingProcess/cac:ContractingSystem[cbc:ContractingSystemTypeCode/@listName='dps-usage']/cbc:ContractingSystemTypeCode/@listName</t>
+  </si>
+  <si>
+    <t>not(cbc:ContractingSystemTypeCode/text()='none')</t>
   </si>
   <si>
     <t>?this epo:foreseesTechnique / epo:hasDPSScope ?value .   FILTER ( ISIRI(?value) &amp;&amp; CONTAINS(str(?value), 'europa.eu/') )</t>
@@ -68872,13 +68875,13 @@
         <v>5072</v>
       </c>
       <c r="H1432" s="32" t="s">
-        <v>946</v>
+        <v>5073</v>
       </c>
       <c r="I1432" s="32" t="s">
         <v>3671</v>
       </c>
       <c r="J1432" s="32" t="s">
-        <v>5073</v>
+        <v>5074</v>
       </c>
       <c r="K1432" s="31"/>
       <c r="L1432" s="29"/>
@@ -68893,10 +68896,10 @@
       <c r="A1433" s="29"/>
       <c r="B1433" s="29"/>
       <c r="C1433" s="30" t="s">
-        <v>5074</v>
+        <v>5075</v>
       </c>
       <c r="D1433" s="32" t="s">
-        <v>5075</v>
+        <v>5076</v>
       </c>
       <c r="E1433" s="32" t="s">
         <v>1413</v>
@@ -68905,7 +68908,7 @@
         <v>910</v>
       </c>
       <c r="G1433" s="32" t="s">
-        <v>5076</v>
+        <v>5077</v>
       </c>
       <c r="H1433" s="32" t="s">
         <v>1415</v>
@@ -68914,7 +68917,7 @@
         <v>1416</v>
       </c>
       <c r="J1433" s="32" t="s">
-        <v>5077</v>
+        <v>5078</v>
       </c>
       <c r="K1433" s="31"/>
       <c r="L1433" s="29"/>
@@ -68929,10 +68932,10 @@
       <c r="A1434" s="29"/>
       <c r="B1434" s="29"/>
       <c r="C1434" s="30" t="s">
-        <v>5078</v>
+        <v>5079</v>
       </c>
       <c r="D1434" s="32" t="s">
-        <v>5079</v>
+        <v>5080</v>
       </c>
       <c r="E1434" s="32" t="s">
         <v>1554</v>
@@ -68941,14 +68944,14 @@
         <v>658</v>
       </c>
       <c r="G1434" s="32" t="s">
-        <v>5080</v>
+        <v>5081</v>
       </c>
       <c r="H1434" s="31"/>
       <c r="I1434" s="32" t="s">
         <v>813</v>
       </c>
       <c r="J1434" s="32" t="s">
-        <v>5081</v>
+        <v>5082</v>
       </c>
       <c r="K1434" s="31"/>
       <c r="L1434" s="29"/>
@@ -68965,10 +68968,10 @@
         <v>487</v>
       </c>
       <c r="C1435" s="30" t="s">
-        <v>5082</v>
+        <v>5083</v>
       </c>
       <c r="D1435" s="32" t="s">
-        <v>5083</v>
+        <v>5084</v>
       </c>
       <c r="E1435" s="32" t="s">
         <v>1375</v>
@@ -68977,14 +68980,14 @@
         <v>910</v>
       </c>
       <c r="G1435" s="32" t="s">
-        <v>5084</v>
+        <v>5085</v>
       </c>
       <c r="H1435" s="31"/>
       <c r="I1435" s="32" t="s">
         <v>1377</v>
       </c>
       <c r="J1435" s="32" t="s">
-        <v>5085</v>
+        <v>5086</v>
       </c>
       <c r="K1435" s="31"/>
       <c r="L1435" s="29"/>
@@ -69003,10 +69006,10 @@
         <v>487</v>
       </c>
       <c r="C1436" s="30" t="s">
-        <v>5086</v>
+        <v>5087</v>
       </c>
       <c r="D1436" s="32" t="s">
-        <v>5087</v>
+        <v>5088</v>
       </c>
       <c r="E1436" s="32" t="s">
         <v>1381</v>
@@ -69015,7 +69018,7 @@
         <v>910</v>
       </c>
       <c r="G1436" s="32" t="s">
-        <v>5088</v>
+        <v>5089</v>
       </c>
       <c r="H1436" s="32" t="s">
         <v>1383</v>
@@ -69024,7 +69027,7 @@
         <v>1384</v>
       </c>
       <c r="J1436" s="32" t="s">
-        <v>5089</v>
+        <v>5090</v>
       </c>
       <c r="K1436" s="31"/>
       <c r="L1436" s="29"/>
@@ -69041,10 +69044,10 @@
       <c r="A1437" s="29"/>
       <c r="B1437" s="29"/>
       <c r="C1437" s="30" t="s">
-        <v>5090</v>
+        <v>5091</v>
       </c>
       <c r="D1437" s="32" t="s">
-        <v>5091</v>
+        <v>5092</v>
       </c>
       <c r="E1437" s="32" t="s">
         <v>2910</v>
@@ -69053,7 +69056,7 @@
         <v>2727</v>
       </c>
       <c r="G1437" s="32" t="s">
-        <v>5092</v>
+        <v>5093</v>
       </c>
       <c r="H1437" s="32" t="s">
         <v>2912</v>
@@ -69062,7 +69065,7 @@
         <v>2913</v>
       </c>
       <c r="J1437" s="32" t="s">
-        <v>5093</v>
+        <v>5094</v>
       </c>
       <c r="K1437" s="31"/>
       <c r="L1437" s="29"/>
@@ -69077,10 +69080,10 @@
       <c r="A1438" s="29"/>
       <c r="B1438" s="29"/>
       <c r="C1438" s="30" t="s">
-        <v>5094</v>
+        <v>5095</v>
       </c>
       <c r="D1438" s="32" t="s">
-        <v>5095</v>
+        <v>5096</v>
       </c>
       <c r="E1438" s="32" t="s">
         <v>710</v>
@@ -69089,14 +69092,14 @@
         <v>711</v>
       </c>
       <c r="G1438" s="32" t="s">
-        <v>5096</v>
+        <v>5097</v>
       </c>
       <c r="H1438" s="31"/>
       <c r="I1438" s="32" t="s">
         <v>713</v>
       </c>
       <c r="J1438" s="32" t="s">
-        <v>5097</v>
+        <v>5098</v>
       </c>
       <c r="K1438" s="31"/>
       <c r="L1438" s="29"/>
@@ -69111,10 +69114,10 @@
       <c r="A1439" s="29"/>
       <c r="B1439" s="29"/>
       <c r="C1439" s="30" t="s">
-        <v>5098</v>
+        <v>5099</v>
       </c>
       <c r="D1439" s="32" t="s">
-        <v>5099</v>
+        <v>5100</v>
       </c>
       <c r="E1439" s="32" t="s">
         <v>724</v>
@@ -69123,14 +69126,14 @@
         <v>725</v>
       </c>
       <c r="G1439" s="32" t="s">
-        <v>5100</v>
+        <v>5101</v>
       </c>
       <c r="H1439" s="31"/>
       <c r="I1439" s="32" t="s">
         <v>727</v>
       </c>
       <c r="J1439" s="32" t="s">
-        <v>5097</v>
+        <v>5098</v>
       </c>
       <c r="K1439" s="31"/>
       <c r="L1439" s="29"/>
@@ -69145,10 +69148,10 @@
       <c r="A1440" s="29"/>
       <c r="B1440" s="29"/>
       <c r="C1440" s="30" t="s">
-        <v>5101</v>
+        <v>5102</v>
       </c>
       <c r="D1440" s="32" t="s">
-        <v>5102</v>
+        <v>5103</v>
       </c>
       <c r="E1440" s="32" t="s">
         <v>730</v>
@@ -69157,14 +69160,14 @@
         <v>731</v>
       </c>
       <c r="G1440" s="32" t="s">
-        <v>5103</v>
+        <v>5104</v>
       </c>
       <c r="H1440" s="31"/>
       <c r="I1440" s="32" t="s">
         <v>733</v>
       </c>
       <c r="J1440" s="32" t="s">
-        <v>5097</v>
+        <v>5098</v>
       </c>
       <c r="K1440" s="31"/>
       <c r="L1440" s="29"/>
@@ -69179,10 +69182,10 @@
       <c r="A1441" s="29"/>
       <c r="B1441" s="29"/>
       <c r="C1441" s="30" t="s">
-        <v>5104</v>
+        <v>5105</v>
       </c>
       <c r="D1441" s="32" t="s">
-        <v>5105</v>
+        <v>5106</v>
       </c>
       <c r="E1441" s="32" t="s">
         <v>750</v>
@@ -69191,14 +69194,14 @@
         <v>751</v>
       </c>
       <c r="G1441" s="32" t="s">
-        <v>5106</v>
+        <v>5107</v>
       </c>
       <c r="H1441" s="31"/>
       <c r="I1441" s="32" t="s">
         <v>753</v>
       </c>
       <c r="J1441" s="32" t="s">
-        <v>5107</v>
+        <v>5108</v>
       </c>
       <c r="K1441" s="31"/>
       <c r="L1441" s="29"/>
@@ -69215,26 +69218,26 @@
         <v>487</v>
       </c>
       <c r="C1442" s="30" t="s">
-        <v>5108</v>
+        <v>5109</v>
       </c>
       <c r="D1442" s="32" t="s">
-        <v>5109</v>
+        <v>5110</v>
       </c>
       <c r="E1442" s="32" t="s">
-        <v>5110</v>
+        <v>5111</v>
       </c>
       <c r="F1442" s="32" t="s">
-        <v>5111</v>
+        <v>5112</v>
       </c>
       <c r="G1442" s="32" t="s">
-        <v>5112</v>
+        <v>5113</v>
       </c>
       <c r="H1442" s="31"/>
       <c r="I1442" s="32" t="s">
-        <v>5113</v>
+        <v>5114</v>
       </c>
       <c r="J1442" s="32" t="s">
-        <v>5114</v>
+        <v>5115</v>
       </c>
       <c r="K1442" s="31"/>
       <c r="L1442" s="29"/>
@@ -69251,26 +69254,26 @@
       <c r="A1443" s="29"/>
       <c r="B1443" s="29"/>
       <c r="C1443" s="30" t="s">
-        <v>5115</v>
+        <v>5116</v>
       </c>
       <c r="D1443" s="32" t="s">
-        <v>5116</v>
+        <v>5117</v>
       </c>
       <c r="E1443" s="32" t="s">
-        <v>5117</v>
+        <v>5118</v>
       </c>
       <c r="F1443" s="32" t="s">
-        <v>5118</v>
+        <v>5119</v>
       </c>
       <c r="G1443" s="32" t="s">
-        <v>5119</v>
+        <v>5120</v>
       </c>
       <c r="H1443" s="31"/>
       <c r="I1443" s="32" t="s">
-        <v>5120</v>
+        <v>5121</v>
       </c>
       <c r="J1443" s="32" t="s">
-        <v>5121</v>
+        <v>5122</v>
       </c>
       <c r="K1443" s="31"/>
       <c r="L1443" s="29"/>
@@ -69285,26 +69288,26 @@
       <c r="A1444" s="29"/>
       <c r="B1444" s="29"/>
       <c r="C1444" s="30" t="s">
-        <v>5122</v>
+        <v>5123</v>
       </c>
       <c r="D1444" s="32" t="s">
-        <v>5123</v>
+        <v>5124</v>
       </c>
       <c r="E1444" s="32" t="s">
-        <v>5124</v>
+        <v>5125</v>
       </c>
       <c r="F1444" s="32" t="s">
         <v>658</v>
       </c>
       <c r="G1444" s="32" t="s">
-        <v>5125</v>
+        <v>5126</v>
       </c>
       <c r="H1444" s="31"/>
       <c r="I1444" s="32" t="s">
         <v>813</v>
       </c>
       <c r="J1444" s="32" t="s">
-        <v>5126</v>
+        <v>5127</v>
       </c>
       <c r="K1444" s="31"/>
       <c r="L1444" s="29"/>
@@ -69321,26 +69324,26 @@
         <v>487</v>
       </c>
       <c r="C1445" s="30" t="s">
-        <v>5127</v>
+        <v>5128</v>
       </c>
       <c r="D1445" s="32" t="s">
-        <v>5128</v>
+        <v>5129</v>
       </c>
       <c r="E1445" s="32" t="s">
-        <v>5129</v>
+        <v>5130</v>
       </c>
       <c r="F1445" s="32" t="s">
-        <v>5130</v>
+        <v>5131</v>
       </c>
       <c r="G1445" s="32" t="s">
-        <v>5131</v>
+        <v>5132</v>
       </c>
       <c r="H1445" s="31"/>
       <c r="I1445" s="32" t="s">
-        <v>5113</v>
+        <v>5114</v>
       </c>
       <c r="J1445" s="32" t="s">
-        <v>5132</v>
+        <v>5133</v>
       </c>
       <c r="K1445" s="31"/>
       <c r="L1445" s="29"/>
@@ -69359,17 +69362,17 @@
         <v>164</v>
       </c>
       <c r="C1446" s="30" t="s">
-        <v>5133</v>
+        <v>5134</v>
       </c>
       <c r="D1446" s="32" t="s">
-        <v>5134</v>
+        <v>5135</v>
       </c>
       <c r="E1446" s="32" t="s">
-        <v>5135</v>
+        <v>5136</v>
       </c>
       <c r="F1446" s="32"/>
       <c r="G1446" s="32" t="s">
-        <v>5136</v>
+        <v>5137</v>
       </c>
       <c r="H1446" s="31"/>
       <c r="I1446" s="32"/>
@@ -69391,25 +69394,25 @@
         <v>164</v>
       </c>
       <c r="C1447" s="30" t="s">
-        <v>5137</v>
+        <v>5138</v>
       </c>
       <c r="D1447" s="32" t="s">
-        <v>5138</v>
+        <v>5139</v>
       </c>
       <c r="E1447" s="32" t="s">
-        <v>5139</v>
+        <v>5140</v>
       </c>
       <c r="F1447" s="32" t="s">
-        <v>5140</v>
+        <v>5141</v>
       </c>
       <c r="G1447" s="32" t="s">
-        <v>5141</v>
+        <v>5142</v>
       </c>
       <c r="H1447" s="32" t="s">
-        <v>5142</v>
+        <v>5143</v>
       </c>
       <c r="I1447" s="32" t="s">
-        <v>5143</v>
+        <v>5144</v>
       </c>
       <c r="J1447" s="32" t="s">
         <v>4649</v>
@@ -69431,25 +69434,25 @@
         <v>164</v>
       </c>
       <c r="C1448" s="30" t="s">
+        <v>5145</v>
+      </c>
+      <c r="D1448" s="32" t="s">
+        <v>5146</v>
+      </c>
+      <c r="E1448" s="32" t="s">
+        <v>5147</v>
+      </c>
+      <c r="F1448" s="32" t="s">
+        <v>5141</v>
+      </c>
+      <c r="G1448" s="32" t="s">
+        <v>5148</v>
+      </c>
+      <c r="H1448" s="32" t="s">
+        <v>5143</v>
+      </c>
+      <c r="I1448" s="32" t="s">
         <v>5144</v>
-      </c>
-      <c r="D1448" s="32" t="s">
-        <v>5145</v>
-      </c>
-      <c r="E1448" s="32" t="s">
-        <v>5146</v>
-      </c>
-      <c r="F1448" s="32" t="s">
-        <v>5140</v>
-      </c>
-      <c r="G1448" s="32" t="s">
-        <v>5147</v>
-      </c>
-      <c r="H1448" s="32" t="s">
-        <v>5142</v>
-      </c>
-      <c r="I1448" s="32" t="s">
-        <v>5143</v>
       </c>
       <c r="J1448" s="32" t="s">
         <v>4086</v>
@@ -69469,10 +69472,10 @@
       <c r="A1449" s="29"/>
       <c r="B1449" s="29"/>
       <c r="C1449" s="30" t="s">
-        <v>5148</v>
+        <v>5149</v>
       </c>
       <c r="D1449" s="32" t="s">
-        <v>5149</v>
+        <v>5150</v>
       </c>
       <c r="E1449" s="32" t="s">
         <v>1445</v>
@@ -69481,14 +69484,14 @@
         <v>658</v>
       </c>
       <c r="G1449" s="32" t="s">
-        <v>5150</v>
+        <v>5151</v>
       </c>
       <c r="H1449" s="31"/>
       <c r="I1449" s="32" t="s">
         <v>1447</v>
       </c>
       <c r="J1449" s="32" t="s">
-        <v>5151</v>
+        <v>5152</v>
       </c>
       <c r="K1449" s="31"/>
       <c r="L1449" s="29"/>
@@ -69505,26 +69508,26 @@
         <v>164</v>
       </c>
       <c r="C1450" s="30" t="s">
-        <v>5152</v>
+        <v>5153</v>
       </c>
       <c r="D1450" s="32" t="s">
-        <v>5153</v>
+        <v>5154</v>
       </c>
       <c r="E1450" s="32" t="s">
-        <v>5154</v>
+        <v>5155</v>
       </c>
       <c r="F1450" s="32" t="s">
-        <v>5140</v>
+        <v>5141</v>
       </c>
       <c r="G1450" s="32" t="s">
-        <v>5155</v>
+        <v>5156</v>
       </c>
       <c r="H1450" s="31"/>
       <c r="I1450" s="32" t="s">
-        <v>5156</v>
+        <v>5157</v>
       </c>
       <c r="J1450" s="32" t="s">
-        <v>5157</v>
+        <v>5158</v>
       </c>
       <c r="K1450" s="31"/>
       <c r="L1450" s="29"/>
@@ -69543,28 +69546,28 @@
         <v>164</v>
       </c>
       <c r="C1451" s="30" t="s">
-        <v>5158</v>
+        <v>5159</v>
       </c>
       <c r="D1451" s="32" t="s">
-        <v>5159</v>
+        <v>5160</v>
       </c>
       <c r="E1451" s="32" t="s">
-        <v>5160</v>
+        <v>5161</v>
       </c>
       <c r="F1451" s="32" t="s">
-        <v>5140</v>
+        <v>5141</v>
       </c>
       <c r="G1451" s="32" t="s">
-        <v>5161</v>
+        <v>5162</v>
       </c>
       <c r="H1451" s="32" t="s">
-        <v>5162</v>
+        <v>5163</v>
       </c>
       <c r="I1451" s="32" t="s">
-        <v>5163</v>
+        <v>5164</v>
       </c>
       <c r="J1451" s="32" t="s">
-        <v>5164</v>
+        <v>5165</v>
       </c>
       <c r="K1451" s="31"/>
       <c r="L1451" s="29"/>
@@ -69583,28 +69586,28 @@
         <v>164</v>
       </c>
       <c r="C1452" s="30" t="s">
-        <v>5165</v>
+        <v>5166</v>
       </c>
       <c r="D1452" s="32" t="s">
-        <v>5166</v>
+        <v>5167</v>
       </c>
       <c r="E1452" s="32" t="s">
-        <v>5167</v>
+        <v>5168</v>
       </c>
       <c r="F1452" s="32" t="s">
-        <v>5140</v>
+        <v>5141</v>
       </c>
       <c r="G1452" s="32" t="s">
-        <v>5168</v>
+        <v>5169</v>
       </c>
       <c r="H1452" s="32" t="s">
-        <v>5162</v>
+        <v>5163</v>
       </c>
       <c r="I1452" s="32" t="s">
-        <v>5169</v>
+        <v>5170</v>
       </c>
       <c r="J1452" s="32" t="s">
-        <v>5170</v>
+        <v>5171</v>
       </c>
       <c r="K1452" s="31"/>
       <c r="L1452" s="29"/>
@@ -69623,26 +69626,26 @@
         <v>487</v>
       </c>
       <c r="C1453" s="30" t="s">
-        <v>5171</v>
+        <v>5172</v>
       </c>
       <c r="D1453" s="32" t="s">
-        <v>5172</v>
+        <v>5173</v>
       </c>
       <c r="E1453" s="32" t="s">
-        <v>5173</v>
+        <v>5174</v>
       </c>
       <c r="F1453" s="32" t="s">
-        <v>5174</v>
+        <v>5175</v>
       </c>
       <c r="G1453" s="32" t="s">
-        <v>5175</v>
+        <v>5176</v>
       </c>
       <c r="H1453" s="31"/>
       <c r="I1453" s="32" t="s">
-        <v>5176</v>
+        <v>5177</v>
       </c>
       <c r="J1453" s="32" t="s">
-        <v>5177</v>
+        <v>5178</v>
       </c>
       <c r="K1453" s="31"/>
       <c r="L1453" s="29"/>
@@ -69661,28 +69664,28 @@
         <v>487</v>
       </c>
       <c r="C1454" s="30" t="s">
-        <v>5178</v>
+        <v>5179</v>
       </c>
       <c r="D1454" s="32" t="s">
-        <v>5179</v>
+        <v>5180</v>
       </c>
       <c r="E1454" s="32" t="s">
-        <v>5180</v>
+        <v>5181</v>
       </c>
       <c r="F1454" s="32" t="s">
-        <v>5181</v>
+        <v>5182</v>
       </c>
       <c r="G1454" s="32" t="s">
-        <v>5182</v>
+        <v>5183</v>
       </c>
       <c r="H1454" s="32" t="s">
-        <v>5183</v>
+        <v>5184</v>
       </c>
       <c r="I1454" s="32" t="s">
-        <v>5184</v>
+        <v>5185</v>
       </c>
       <c r="J1454" s="32" t="s">
-        <v>5185</v>
+        <v>5186</v>
       </c>
       <c r="K1454" s="31"/>
       <c r="L1454" s="29"/>
@@ -69701,28 +69704,28 @@
         <v>164</v>
       </c>
       <c r="C1455" s="30" t="s">
-        <v>5186</v>
+        <v>5187</v>
       </c>
       <c r="D1455" s="32" t="s">
-        <v>5187</v>
+        <v>5188</v>
       </c>
       <c r="E1455" s="32" t="s">
-        <v>5188</v>
+        <v>5189</v>
       </c>
       <c r="F1455" s="32" t="s">
-        <v>5140</v>
+        <v>5141</v>
       </c>
       <c r="G1455" s="32" t="s">
-        <v>5189</v>
+        <v>5190</v>
       </c>
       <c r="H1455" s="32" t="s">
-        <v>5142</v>
+        <v>5143</v>
       </c>
       <c r="I1455" s="32" t="s">
-        <v>5143</v>
+        <v>5144</v>
       </c>
       <c r="J1455" s="32" t="s">
-        <v>5190</v>
+        <v>5191</v>
       </c>
       <c r="K1455" s="31"/>
       <c r="L1455" s="29"/>
@@ -69741,26 +69744,26 @@
         <v>164</v>
       </c>
       <c r="C1456" s="30" t="s">
-        <v>5191</v>
+        <v>5192</v>
       </c>
       <c r="D1456" s="32" t="s">
-        <v>5192</v>
+        <v>5193</v>
       </c>
       <c r="E1456" s="32" t="s">
-        <v>5193</v>
+        <v>5194</v>
       </c>
       <c r="F1456" s="32" t="s">
-        <v>5194</v>
+        <v>5195</v>
       </c>
       <c r="G1456" s="32" t="s">
-        <v>5195</v>
+        <v>5196</v>
       </c>
       <c r="H1456" s="31"/>
       <c r="I1456" s="32" t="s">
-        <v>5196</v>
+        <v>5197</v>
       </c>
       <c r="J1456" s="32" t="s">
-        <v>5197</v>
+        <v>5198</v>
       </c>
       <c r="K1456" s="31"/>
       <c r="L1456" s="29"/>
@@ -69777,26 +69780,26 @@
       <c r="A1457" s="29"/>
       <c r="B1457" s="29"/>
       <c r="C1457" s="30" t="s">
-        <v>5198</v>
+        <v>5199</v>
       </c>
       <c r="D1457" s="32" t="s">
-        <v>5199</v>
+        <v>5200</v>
       </c>
       <c r="E1457" s="32" t="s">
-        <v>5200</v>
+        <v>5201</v>
       </c>
       <c r="F1457" s="32" t="s">
-        <v>5201</v>
+        <v>5202</v>
       </c>
       <c r="G1457" s="32" t="s">
-        <v>5202</v>
+        <v>5203</v>
       </c>
       <c r="H1457" s="31"/>
       <c r="I1457" s="32" t="s">
-        <v>5203</v>
+        <v>5204</v>
       </c>
       <c r="J1457" s="32" t="s">
-        <v>5204</v>
+        <v>5205</v>
       </c>
       <c r="K1457" s="31"/>
       <c r="L1457" s="29"/>
@@ -69811,23 +69814,23 @@
       <c r="A1458" s="29"/>
       <c r="B1458" s="29"/>
       <c r="C1458" s="30" t="s">
-        <v>5205</v>
+        <v>5206</v>
       </c>
       <c r="D1458" s="32" t="s">
-        <v>5206</v>
+        <v>5207</v>
       </c>
       <c r="E1458" s="32" t="s">
-        <v>5207</v>
+        <v>5208</v>
       </c>
       <c r="F1458" s="32" t="s">
-        <v>5201</v>
+        <v>5202</v>
       </c>
       <c r="G1458" s="32" t="s">
-        <v>5208</v>
+        <v>5209</v>
       </c>
       <c r="H1458" s="31"/>
       <c r="I1458" s="32" t="s">
-        <v>5209</v>
+        <v>5210</v>
       </c>
       <c r="J1458" s="32" t="s">
         <v>4960</v>
@@ -69845,10 +69848,10 @@
       <c r="A1459" s="29"/>
       <c r="B1459" s="29"/>
       <c r="C1459" s="30" t="s">
-        <v>5210</v>
+        <v>5211</v>
       </c>
       <c r="D1459" s="32" t="s">
-        <v>5211</v>
+        <v>5212</v>
       </c>
       <c r="E1459" s="32" t="s">
         <v>719</v>
@@ -69857,14 +69860,14 @@
         <v>711</v>
       </c>
       <c r="G1459" s="32" t="s">
-        <v>5212</v>
+        <v>5213</v>
       </c>
       <c r="H1459" s="31"/>
       <c r="I1459" s="32" t="s">
         <v>721</v>
       </c>
       <c r="J1459" s="32" t="s">
-        <v>5097</v>
+        <v>5098</v>
       </c>
       <c r="K1459" s="31"/>
       <c r="L1459" s="29"/>
@@ -69879,10 +69882,10 @@
       <c r="A1460" s="29"/>
       <c r="B1460" s="29"/>
       <c r="C1460" s="30" t="s">
-        <v>5213</v>
+        <v>5214</v>
       </c>
       <c r="D1460" s="32" t="s">
-        <v>5214</v>
+        <v>5215</v>
       </c>
       <c r="E1460" s="32" t="s">
         <v>551</v>
@@ -69891,7 +69894,7 @@
         <v>294</v>
       </c>
       <c r="G1460" s="32" t="s">
-        <v>5215</v>
+        <v>5216</v>
       </c>
       <c r="H1460" s="32" t="s">
         <v>553</v>
@@ -69900,7 +69903,7 @@
         <v>350</v>
       </c>
       <c r="J1460" s="32" t="s">
-        <v>5216</v>
+        <v>5217</v>
       </c>
       <c r="K1460" s="31"/>
       <c r="L1460" s="29"/>
@@ -69915,10 +69918,10 @@
       <c r="A1461" s="29"/>
       <c r="B1461" s="29"/>
       <c r="C1461" s="30" t="s">
-        <v>5217</v>
+        <v>5218</v>
       </c>
       <c r="D1461" s="32" t="s">
-        <v>5218</v>
+        <v>5219</v>
       </c>
       <c r="E1461" s="32" t="s">
         <v>1408</v>
@@ -69927,14 +69930,14 @@
         <v>595</v>
       </c>
       <c r="G1461" s="32" t="s">
-        <v>5219</v>
+        <v>5220</v>
       </c>
       <c r="H1461" s="31"/>
       <c r="I1461" s="32" t="s">
         <v>654</v>
       </c>
       <c r="J1461" s="32" t="s">
-        <v>5220</v>
+        <v>5221</v>
       </c>
       <c r="K1461" s="31"/>
       <c r="L1461" s="29"/>
@@ -69949,10 +69952,10 @@
       <c r="A1462" s="29"/>
       <c r="B1462" s="29"/>
       <c r="C1462" s="30" t="s">
-        <v>5221</v>
+        <v>5222</v>
       </c>
       <c r="D1462" s="32" t="s">
-        <v>5222</v>
+        <v>5223</v>
       </c>
       <c r="E1462" s="32" t="s">
         <v>931</v>
@@ -69961,14 +69964,14 @@
         <v>1669</v>
       </c>
       <c r="G1462" s="32" t="s">
-        <v>5223</v>
+        <v>5224</v>
       </c>
       <c r="H1462" s="31"/>
       <c r="I1462" s="32" t="s">
         <v>1673</v>
       </c>
       <c r="J1462" s="32" t="s">
-        <v>5224</v>
+        <v>5225</v>
       </c>
       <c r="K1462" s="31"/>
       <c r="L1462" s="29"/>
@@ -69983,10 +69986,10 @@
       <c r="A1463" s="29"/>
       <c r="B1463" s="29"/>
       <c r="C1463" s="30" t="s">
-        <v>5225</v>
+        <v>5226</v>
       </c>
       <c r="D1463" s="32" t="s">
-        <v>5226</v>
+        <v>5227</v>
       </c>
       <c r="E1463" s="32" t="s">
         <v>1880</v>
@@ -69995,14 +69998,14 @@
         <v>1875</v>
       </c>
       <c r="G1463" s="32" t="s">
-        <v>5227</v>
+        <v>5228</v>
       </c>
       <c r="H1463" s="31"/>
       <c r="I1463" s="32" t="s">
         <v>1882</v>
       </c>
       <c r="J1463" s="32" t="s">
-        <v>5228</v>
+        <v>5229</v>
       </c>
       <c r="K1463" s="31"/>
       <c r="L1463" s="29"/>
@@ -70017,10 +70020,10 @@
       <c r="A1464" s="29"/>
       <c r="B1464" s="29"/>
       <c r="C1464" s="30" t="s">
-        <v>5229</v>
+        <v>5230</v>
       </c>
       <c r="D1464" s="32" t="s">
-        <v>5230</v>
+        <v>5231</v>
       </c>
       <c r="E1464" s="32" t="s">
         <v>184</v>
@@ -70029,7 +70032,7 @@
         <v>42</v>
       </c>
       <c r="G1464" s="32" t="s">
-        <v>5231</v>
+        <v>5232</v>
       </c>
       <c r="H1464" s="31"/>
       <c r="I1464" s="32" t="s">
@@ -70051,10 +70054,10 @@
       <c r="A1465" s="29"/>
       <c r="B1465" s="29"/>
       <c r="C1465" s="30" t="s">
-        <v>5232</v>
+        <v>5233</v>
       </c>
       <c r="D1465" s="32" t="s">
-        <v>5233</v>
+        <v>5234</v>
       </c>
       <c r="E1465" s="32" t="s">
         <v>189</v>
@@ -70063,7 +70066,7 @@
         <v>42</v>
       </c>
       <c r="G1465" s="32" t="s">
-        <v>5234</v>
+        <v>5235</v>
       </c>
       <c r="H1465" s="31"/>
       <c r="I1465" s="32" t="s">
@@ -70085,10 +70088,10 @@
       <c r="A1466" s="29"/>
       <c r="B1466" s="29"/>
       <c r="C1466" s="30" t="s">
-        <v>5235</v>
+        <v>5236</v>
       </c>
       <c r="D1466" s="32" t="s">
-        <v>5236</v>
+        <v>5237</v>
       </c>
       <c r="E1466" s="32" t="s">
         <v>4013</v>
@@ -70097,14 +70100,14 @@
         <v>4014</v>
       </c>
       <c r="G1466" s="32" t="s">
-        <v>5237</v>
+        <v>5238</v>
       </c>
       <c r="H1466" s="31"/>
       <c r="I1466" s="32" t="s">
-        <v>5238</v>
+        <v>5239</v>
       </c>
       <c r="J1466" s="32" t="s">
-        <v>5239</v>
+        <v>5240</v>
       </c>
       <c r="K1466" s="31"/>
       <c r="L1466" s="29"/>
@@ -70119,17 +70122,17 @@
       <c r="A1467" s="29"/>
       <c r="B1467" s="29"/>
       <c r="C1467" s="30" t="s">
-        <v>5240</v>
+        <v>5241</v>
       </c>
       <c r="D1467" s="32" t="s">
-        <v>5241</v>
+        <v>5242</v>
       </c>
       <c r="E1467" s="32" t="s">
         <v>4051</v>
       </c>
       <c r="F1467" s="32"/>
       <c r="G1467" s="32" t="s">
-        <v>5242</v>
+        <v>5243</v>
       </c>
       <c r="H1467" s="31"/>
       <c r="I1467" s="32"/>
@@ -70147,10 +70150,10 @@
       <c r="A1468" s="29"/>
       <c r="B1468" s="29"/>
       <c r="C1468" s="30" t="s">
-        <v>5243</v>
+        <v>5244</v>
       </c>
       <c r="D1468" s="32" t="s">
-        <v>5244</v>
+        <v>5245</v>
       </c>
       <c r="E1468" s="32" t="s">
         <v>4056</v>
@@ -70159,7 +70162,7 @@
         <v>476</v>
       </c>
       <c r="G1468" s="32" t="s">
-        <v>5245</v>
+        <v>5246</v>
       </c>
       <c r="H1468" s="32" t="s">
         <v>4058</v>
@@ -70168,7 +70171,7 @@
         <v>485</v>
       </c>
       <c r="J1468" s="32" t="s">
-        <v>5246</v>
+        <v>5247</v>
       </c>
       <c r="K1468" s="31"/>
       <c r="L1468" s="29"/>
@@ -70183,17 +70186,17 @@
       <c r="A1469" s="29"/>
       <c r="B1469" s="29"/>
       <c r="C1469" s="30" t="s">
-        <v>5247</v>
+        <v>5248</v>
       </c>
       <c r="D1469" s="32" t="s">
-        <v>5248</v>
+        <v>5249</v>
       </c>
       <c r="E1469" s="32" t="s">
         <v>4072</v>
       </c>
       <c r="F1469" s="32"/>
       <c r="G1469" s="32" t="s">
-        <v>5249</v>
+        <v>5250</v>
       </c>
       <c r="H1469" s="31"/>
       <c r="I1469" s="32"/>
@@ -70211,10 +70214,10 @@
       <c r="A1470" s="29"/>
       <c r="B1470" s="29"/>
       <c r="C1470" s="30" t="s">
-        <v>5250</v>
+        <v>5251</v>
       </c>
       <c r="D1470" s="32" t="s">
-        <v>5251</v>
+        <v>5252</v>
       </c>
       <c r="E1470" s="32" t="s">
         <v>4077</v>
@@ -70223,14 +70226,14 @@
         <v>476</v>
       </c>
       <c r="G1470" s="32" t="s">
-        <v>5252</v>
+        <v>5253</v>
       </c>
       <c r="H1470" s="31"/>
       <c r="I1470" s="32" t="s">
         <v>485</v>
       </c>
       <c r="J1470" s="32" t="s">
-        <v>5253</v>
+        <v>5254</v>
       </c>
       <c r="K1470" s="31"/>
       <c r="L1470" s="29"/>
@@ -70245,10 +70248,10 @@
       <c r="A1471" s="29"/>
       <c r="B1471" s="29"/>
       <c r="C1471" s="30" t="s">
-        <v>5254</v>
+        <v>5255</v>
       </c>
       <c r="D1471" s="32" t="s">
-        <v>5255</v>
+        <v>5256</v>
       </c>
       <c r="E1471" s="32" t="s">
         <v>3969</v>
@@ -70257,14 +70260,14 @@
         <v>3970</v>
       </c>
       <c r="G1471" s="32" t="s">
-        <v>5256</v>
+        <v>5257</v>
       </c>
       <c r="H1471" s="31"/>
       <c r="I1471" s="32" t="s">
         <v>3972</v>
       </c>
       <c r="J1471" s="32" t="s">
-        <v>5257</v>
+        <v>5258</v>
       </c>
       <c r="K1471" s="31"/>
       <c r="L1471" s="29"/>
@@ -70279,10 +70282,10 @@
       <c r="A1472" s="29"/>
       <c r="B1472" s="29"/>
       <c r="C1472" s="30" t="s">
-        <v>5258</v>
+        <v>5259</v>
       </c>
       <c r="D1472" s="32" t="s">
-        <v>5259</v>
+        <v>5260</v>
       </c>
       <c r="E1472" s="32" t="s">
         <v>177</v>
@@ -70291,7 +70294,7 @@
         <v>42</v>
       </c>
       <c r="G1472" s="32" t="s">
-        <v>5260</v>
+        <v>5261</v>
       </c>
       <c r="H1472" s="31"/>
       <c r="I1472" s="32"/>
@@ -70309,10 +70312,10 @@
       <c r="A1473" s="29"/>
       <c r="B1473" s="29"/>
       <c r="C1473" s="30" t="s">
-        <v>5261</v>
+        <v>5262</v>
       </c>
       <c r="D1473" s="32" t="s">
-        <v>5262</v>
+        <v>5263</v>
       </c>
       <c r="E1473" s="32" t="s">
         <v>4031</v>
@@ -70321,11 +70324,11 @@
         <v>4032</v>
       </c>
       <c r="G1473" s="32" t="s">
-        <v>5263</v>
+        <v>5264</v>
       </c>
       <c r="H1473" s="31"/>
       <c r="I1473" s="32" t="s">
-        <v>5264</v>
+        <v>5265</v>
       </c>
       <c r="J1473" s="32" t="s">
         <v>4035</v>
@@ -70343,10 +70346,10 @@
       <c r="A1474" s="29"/>
       <c r="B1474" s="29"/>
       <c r="C1474" s="30" t="s">
-        <v>5265</v>
+        <v>5266</v>
       </c>
       <c r="D1474" s="32" t="s">
-        <v>5266</v>
+        <v>5267</v>
       </c>
       <c r="E1474" s="32" t="s">
         <v>285</v>
@@ -70355,7 +70358,7 @@
         <v>286</v>
       </c>
       <c r="G1474" s="32" t="s">
-        <v>5267</v>
+        <v>5268</v>
       </c>
       <c r="H1474" s="31"/>
       <c r="I1474" s="32" t="s">
@@ -70377,10 +70380,10 @@
       <c r="A1475" s="29"/>
       <c r="B1475" s="29"/>
       <c r="C1475" s="30" t="s">
-        <v>5268</v>
+        <v>5269</v>
       </c>
       <c r="D1475" s="32" t="s">
-        <v>5269</v>
+        <v>5270</v>
       </c>
       <c r="E1475" s="32" t="s">
         <v>274</v>
@@ -70389,7 +70392,7 @@
         <v>275</v>
       </c>
       <c r="G1475" s="32" t="s">
-        <v>5270</v>
+        <v>5271</v>
       </c>
       <c r="H1475" s="32" t="s">
         <v>277</v>
@@ -70409,17 +70412,17 @@
       <c r="A1476" s="29"/>
       <c r="B1476" s="29"/>
       <c r="C1476" s="30" t="s">
-        <v>5271</v>
+        <v>5272</v>
       </c>
       <c r="D1476" s="32" t="s">
-        <v>5272</v>
+        <v>5273</v>
       </c>
       <c r="E1476" s="32" t="s">
-        <v>5273</v>
+        <v>5274</v>
       </c>
       <c r="F1476" s="32"/>
       <c r="G1476" s="32" t="s">
-        <v>5274</v>
+        <v>5275</v>
       </c>
       <c r="H1476" s="31"/>
       <c r="I1476" s="32"/>
@@ -70437,10 +70440,10 @@
       <c r="A1477" s="29"/>
       <c r="B1477" s="29"/>
       <c r="C1477" s="30" t="s">
-        <v>5275</v>
+        <v>5276</v>
       </c>
       <c r="D1477" s="32" t="s">
-        <v>5276</v>
+        <v>5277</v>
       </c>
       <c r="E1477" s="32" t="s">
         <v>3961</v>
@@ -70449,14 +70452,14 @@
         <v>3962</v>
       </c>
       <c r="G1477" s="32" t="s">
-        <v>5277</v>
+        <v>5278</v>
       </c>
       <c r="H1477" s="31"/>
       <c r="I1477" s="32" t="s">
         <v>813</v>
       </c>
       <c r="J1477" s="32" t="s">
-        <v>5278</v>
+        <v>5279</v>
       </c>
       <c r="K1477" s="31"/>
       <c r="L1477" s="29"/>
@@ -70471,10 +70474,10 @@
       <c r="A1478" s="29"/>
       <c r="B1478" s="29"/>
       <c r="C1478" s="30" t="s">
-        <v>5279</v>
+        <v>5280</v>
       </c>
       <c r="D1478" s="32" t="s">
-        <v>5280</v>
+        <v>5281</v>
       </c>
       <c r="E1478" s="32" t="s">
         <v>3983</v>
@@ -70483,14 +70486,14 @@
         <v>3984</v>
       </c>
       <c r="G1478" s="32" t="s">
-        <v>5281</v>
+        <v>5282</v>
       </c>
       <c r="H1478" s="31"/>
       <c r="I1478" s="32" t="s">
         <v>3986</v>
       </c>
       <c r="J1478" s="32" t="s">
-        <v>5282</v>
+        <v>5283</v>
       </c>
       <c r="K1478" s="31"/>
       <c r="L1478" s="29"/>
@@ -70505,10 +70508,10 @@
       <c r="A1479" s="29"/>
       <c r="B1479" s="29"/>
       <c r="C1479" s="30" t="s">
-        <v>5283</v>
+        <v>5284</v>
       </c>
       <c r="D1479" s="32" t="s">
-        <v>5284</v>
+        <v>5285</v>
       </c>
       <c r="E1479" s="32" t="s">
         <v>3990</v>
@@ -70517,14 +70520,14 @@
         <v>3984</v>
       </c>
       <c r="G1479" s="32" t="s">
-        <v>5285</v>
+        <v>5286</v>
       </c>
       <c r="H1479" s="31"/>
       <c r="I1479" s="32" t="s">
         <v>3992</v>
       </c>
       <c r="J1479" s="32" t="s">
-        <v>5286</v>
+        <v>5287</v>
       </c>
       <c r="K1479" s="31"/>
       <c r="L1479" s="29"/>
@@ -70539,10 +70542,10 @@
       <c r="A1480" s="29"/>
       <c r="B1480" s="29"/>
       <c r="C1480" s="30" t="s">
-        <v>5287</v>
+        <v>5288</v>
       </c>
       <c r="D1480" s="32" t="s">
-        <v>5288</v>
+        <v>5289</v>
       </c>
       <c r="E1480" s="32" t="s">
         <v>2677</v>
@@ -70551,7 +70554,7 @@
         <v>105</v>
       </c>
       <c r="G1480" s="32" t="s">
-        <v>5289</v>
+        <v>5290</v>
       </c>
       <c r="H1480" s="31"/>
       <c r="I1480" s="32" t="s">
@@ -70575,17 +70578,17 @@
         <v>164</v>
       </c>
       <c r="C1481" s="30" t="s">
-        <v>5290</v>
+        <v>5291</v>
       </c>
       <c r="D1481" s="32" t="s">
-        <v>5291</v>
+        <v>5292</v>
       </c>
       <c r="E1481" s="32" t="s">
         <v>3130</v>
       </c>
       <c r="F1481" s="32"/>
       <c r="G1481" s="32" t="s">
-        <v>5292</v>
+        <v>5293</v>
       </c>
       <c r="H1481" s="31"/>
       <c r="I1481" s="32"/>
@@ -70605,10 +70608,10 @@
       <c r="A1482" s="29"/>
       <c r="B1482" s="29"/>
       <c r="C1482" s="30" t="s">
-        <v>5293</v>
+        <v>5294</v>
       </c>
       <c r="D1482" s="32" t="s">
-        <v>5294</v>
+        <v>5295</v>
       </c>
       <c r="E1482" s="32" t="s">
         <v>2123</v>
@@ -70617,7 +70620,7 @@
         <v>2124</v>
       </c>
       <c r="G1482" s="32" t="s">
-        <v>5295</v>
+        <v>5296</v>
       </c>
       <c r="H1482" s="31"/>
       <c r="I1482" s="32" t="s">
@@ -70639,10 +70642,10 @@
       <c r="A1483" s="29"/>
       <c r="B1483" s="29"/>
       <c r="C1483" s="30" t="s">
-        <v>5296</v>
+        <v>5297</v>
       </c>
       <c r="D1483" s="32" t="s">
-        <v>5297</v>
+        <v>5298</v>
       </c>
       <c r="E1483" s="32" t="s">
         <v>2289</v>
@@ -70651,7 +70654,7 @@
         <v>2290</v>
       </c>
       <c r="G1483" s="32" t="s">
-        <v>5298</v>
+        <v>5299</v>
       </c>
       <c r="H1483" s="31"/>
       <c r="I1483" s="32" t="s">
@@ -70673,10 +70676,10 @@
       <c r="A1484" s="29"/>
       <c r="B1484" s="29"/>
       <c r="C1484" s="30" t="s">
-        <v>5299</v>
+        <v>5300</v>
       </c>
       <c r="D1484" s="32" t="s">
-        <v>5300</v>
+        <v>5301</v>
       </c>
       <c r="E1484" s="32" t="s">
         <v>3352</v>
@@ -70685,7 +70688,7 @@
         <v>3353</v>
       </c>
       <c r="G1484" s="32" t="s">
-        <v>5301</v>
+        <v>5302</v>
       </c>
       <c r="H1484" s="31"/>
       <c r="I1484" s="32" t="s">
@@ -70707,17 +70710,17 @@
       <c r="A1485" s="29"/>
       <c r="B1485" s="29"/>
       <c r="C1485" s="30" t="s">
-        <v>5302</v>
+        <v>5303</v>
       </c>
       <c r="D1485" s="32" t="s">
-        <v>5303</v>
+        <v>5304</v>
       </c>
       <c r="E1485" s="32" t="s">
         <v>2558</v>
       </c>
       <c r="F1485" s="32"/>
       <c r="G1485" s="32" t="s">
-        <v>5304</v>
+        <v>5305</v>
       </c>
       <c r="H1485" s="31"/>
       <c r="I1485" s="32"/>
@@ -70735,10 +70738,10 @@
       <c r="A1486" s="29"/>
       <c r="B1486" s="29"/>
       <c r="C1486" s="30" t="s">
-        <v>5305</v>
+        <v>5306</v>
       </c>
       <c r="D1486" s="32" t="s">
-        <v>5306</v>
+        <v>5307</v>
       </c>
       <c r="E1486" s="32" t="s">
         <v>217</v>
@@ -70747,7 +70750,7 @@
         <v>2696</v>
       </c>
       <c r="G1486" s="32" t="s">
-        <v>5307</v>
+        <v>5308</v>
       </c>
       <c r="H1486" s="31"/>
       <c r="I1486" s="32" t="s">
@@ -70771,10 +70774,10 @@
         <v>212</v>
       </c>
       <c r="C1487" s="30" t="s">
-        <v>5308</v>
+        <v>5309</v>
       </c>
       <c r="D1487" s="32" t="s">
-        <v>5309</v>
+        <v>5310</v>
       </c>
       <c r="E1487" s="32" t="s">
         <v>217</v>
@@ -70783,7 +70786,7 @@
         <v>218</v>
       </c>
       <c r="G1487" s="32" t="s">
-        <v>5310</v>
+        <v>5311</v>
       </c>
       <c r="H1487" s="31"/>
       <c r="I1487" s="32" t="s">
@@ -70807,10 +70810,10 @@
       <c r="A1488" s="29"/>
       <c r="B1488" s="29"/>
       <c r="C1488" s="30" t="s">
-        <v>5311</v>
+        <v>5312</v>
       </c>
       <c r="D1488" s="32" t="s">
-        <v>5312</v>
+        <v>5313</v>
       </c>
       <c r="E1488" s="32" t="s">
         <v>217</v>
@@ -70819,7 +70822,7 @@
         <v>269</v>
       </c>
       <c r="G1488" s="32" t="s">
-        <v>5313</v>
+        <v>5314</v>
       </c>
       <c r="H1488" s="31"/>
       <c r="I1488" s="32" t="s">
@@ -70841,10 +70844,10 @@
       <c r="A1489" s="29"/>
       <c r="B1489" s="29"/>
       <c r="C1489" s="30" t="s">
-        <v>5314</v>
+        <v>5315</v>
       </c>
       <c r="D1489" s="32" t="s">
-        <v>5315</v>
+        <v>5316</v>
       </c>
       <c r="E1489" s="32" t="s">
         <v>217</v>
@@ -70853,7 +70856,7 @@
         <v>2567</v>
       </c>
       <c r="G1489" s="32" t="s">
-        <v>5316</v>
+        <v>5317</v>
       </c>
       <c r="H1489" s="32" t="s">
         <v>2569</v>
@@ -70877,10 +70880,10 @@
       <c r="A1490" s="29"/>
       <c r="B1490" s="29"/>
       <c r="C1490" s="30" t="s">
-        <v>5317</v>
+        <v>5318</v>
       </c>
       <c r="D1490" s="32" t="s">
-        <v>5318</v>
+        <v>5319</v>
       </c>
       <c r="E1490" s="32" t="s">
         <v>1020</v>
@@ -70889,7 +70892,7 @@
         <v>1830</v>
       </c>
       <c r="G1490" s="32" t="s">
-        <v>5319</v>
+        <v>5320</v>
       </c>
       <c r="H1490" s="32" t="s">
         <v>204</v>
@@ -70913,10 +70916,10 @@
       <c r="A1491" s="29"/>
       <c r="B1491" s="29"/>
       <c r="C1491" s="30" t="s">
-        <v>5320</v>
+        <v>5321</v>
       </c>
       <c r="D1491" s="32" t="s">
-        <v>5321</v>
+        <v>5322</v>
       </c>
       <c r="E1491" s="32" t="s">
         <v>1020</v>
@@ -70925,7 +70928,7 @@
         <v>1853</v>
       </c>
       <c r="G1491" s="32" t="s">
-        <v>5322</v>
+        <v>5323</v>
       </c>
       <c r="H1491" s="32" t="s">
         <v>204</v>
@@ -70949,10 +70952,10 @@
       <c r="A1492" s="29"/>
       <c r="B1492" s="29"/>
       <c r="C1492" s="30" t="s">
-        <v>5323</v>
+        <v>5324</v>
       </c>
       <c r="D1492" s="32" t="s">
-        <v>5324</v>
+        <v>5325</v>
       </c>
       <c r="E1492" s="32" t="s">
         <v>1020</v>
@@ -70961,7 +70964,7 @@
         <v>1092</v>
       </c>
       <c r="G1492" s="32" t="s">
-        <v>5325</v>
+        <v>5326</v>
       </c>
       <c r="H1492" s="32" t="s">
         <v>1023</v>
@@ -70985,10 +70988,10 @@
       <c r="A1493" s="29"/>
       <c r="B1493" s="29"/>
       <c r="C1493" s="30" t="s">
-        <v>5326</v>
+        <v>5327</v>
       </c>
       <c r="D1493" s="32" t="s">
-        <v>5327</v>
+        <v>5328</v>
       </c>
       <c r="E1493" s="32" t="s">
         <v>1020</v>
@@ -70997,7 +71000,7 @@
         <v>1060</v>
       </c>
       <c r="G1493" s="32" t="s">
-        <v>5328</v>
+        <v>5329</v>
       </c>
       <c r="H1493" s="32" t="s">
         <v>1023</v>
@@ -71021,10 +71024,10 @@
       <c r="A1494" s="29"/>
       <c r="B1494" s="29"/>
       <c r="C1494" s="30" t="s">
-        <v>5329</v>
+        <v>5330</v>
       </c>
       <c r="D1494" s="32" t="s">
-        <v>5330</v>
+        <v>5331</v>
       </c>
       <c r="E1494" s="32" t="s">
         <v>1020</v>
@@ -71033,7 +71036,7 @@
         <v>1021</v>
       </c>
       <c r="G1494" s="32" t="s">
-        <v>5331</v>
+        <v>5332</v>
       </c>
       <c r="H1494" s="32" t="s">
         <v>1023</v>
@@ -71057,10 +71060,10 @@
       <c r="A1495" s="29"/>
       <c r="B1495" s="29"/>
       <c r="C1495" s="30" t="s">
-        <v>5332</v>
+        <v>5333</v>
       </c>
       <c r="D1495" s="32" t="s">
-        <v>5333</v>
+        <v>5334</v>
       </c>
       <c r="E1495" s="32" t="s">
         <v>1020</v>
@@ -71069,7 +71072,7 @@
         <v>1932</v>
       </c>
       <c r="G1495" s="32" t="s">
-        <v>5334</v>
+        <v>5335</v>
       </c>
       <c r="H1495" s="32" t="s">
         <v>204</v>
@@ -71093,10 +71096,10 @@
       <c r="A1496" s="29"/>
       <c r="B1496" s="29"/>
       <c r="C1496" s="30" t="s">
-        <v>5335</v>
+        <v>5336</v>
       </c>
       <c r="D1496" s="32" t="s">
-        <v>5336</v>
+        <v>5337</v>
       </c>
       <c r="E1496" s="32" t="s">
         <v>1020</v>
@@ -71105,7 +71108,7 @@
         <v>1909</v>
       </c>
       <c r="G1496" s="32" t="s">
-        <v>5337</v>
+        <v>5338</v>
       </c>
       <c r="H1496" s="32" t="s">
         <v>204</v>
@@ -71129,10 +71132,10 @@
       <c r="A1497" s="29"/>
       <c r="B1497" s="29"/>
       <c r="C1497" s="30" t="s">
-        <v>5338</v>
+        <v>5339</v>
       </c>
       <c r="D1497" s="32" t="s">
-        <v>5339</v>
+        <v>5340</v>
       </c>
       <c r="E1497" s="32" t="s">
         <v>1020</v>
@@ -71141,7 +71144,7 @@
         <v>1886</v>
       </c>
       <c r="G1497" s="32" t="s">
-        <v>5340</v>
+        <v>5341</v>
       </c>
       <c r="H1497" s="32" t="s">
         <v>204</v>
@@ -71165,10 +71168,10 @@
       <c r="A1498" s="29"/>
       <c r="B1498" s="29"/>
       <c r="C1498" s="30" t="s">
-        <v>5341</v>
+        <v>5342</v>
       </c>
       <c r="D1498" s="32" t="s">
-        <v>5342</v>
+        <v>5343</v>
       </c>
       <c r="E1498" s="32" t="s">
         <v>1020</v>
@@ -71177,7 +71180,7 @@
         <v>1589</v>
       </c>
       <c r="G1498" s="32" t="s">
-        <v>5343</v>
+        <v>5344</v>
       </c>
       <c r="H1498" s="32" t="s">
         <v>204</v>
@@ -71201,10 +71204,10 @@
       <c r="A1499" s="29"/>
       <c r="B1499" s="29"/>
       <c r="C1499" s="30" t="s">
-        <v>5344</v>
+        <v>5345</v>
       </c>
       <c r="D1499" s="32" t="s">
-        <v>5345</v>
+        <v>5346</v>
       </c>
       <c r="E1499" s="32" t="s">
         <v>1020</v>
@@ -71213,7 +71216,7 @@
         <v>1575</v>
       </c>
       <c r="G1499" s="32" t="s">
-        <v>5346</v>
+        <v>5347</v>
       </c>
       <c r="H1499" s="32" t="s">
         <v>1577</v>
@@ -71237,10 +71240,10 @@
       <c r="A1500" s="29"/>
       <c r="B1500" s="29"/>
       <c r="C1500" s="30" t="s">
-        <v>5347</v>
+        <v>5348</v>
       </c>
       <c r="D1500" s="32" t="s">
-        <v>5348</v>
+        <v>5349</v>
       </c>
       <c r="E1500" s="32" t="s">
         <v>1020</v>
@@ -71249,7 +71252,7 @@
         <v>3141</v>
       </c>
       <c r="G1500" s="32" t="s">
-        <v>5349</v>
+        <v>5350</v>
       </c>
       <c r="H1500" s="31"/>
       <c r="I1500" s="32" t="s">
@@ -71271,10 +71274,10 @@
       <c r="A1501" s="29"/>
       <c r="B1501" s="29"/>
       <c r="C1501" s="30" t="s">
-        <v>5350</v>
+        <v>5351</v>
       </c>
       <c r="D1501" s="32" t="s">
-        <v>5351</v>
+        <v>5352</v>
       </c>
       <c r="E1501" s="32" t="s">
         <v>1020</v>
@@ -71283,7 +71286,7 @@
         <v>3147</v>
       </c>
       <c r="G1501" s="32" t="s">
-        <v>5352</v>
+        <v>5353</v>
       </c>
       <c r="H1501" s="31"/>
       <c r="I1501" s="32" t="s">
@@ -71305,10 +71308,10 @@
       <c r="A1502" s="29"/>
       <c r="B1502" s="29"/>
       <c r="C1502" s="30" t="s">
-        <v>5353</v>
+        <v>5354</v>
       </c>
       <c r="D1502" s="32" t="s">
-        <v>5318</v>
+        <v>5319</v>
       </c>
       <c r="E1502" s="32" t="s">
         <v>1020</v>
@@ -71317,7 +71320,7 @@
         <v>3836</v>
       </c>
       <c r="G1502" s="32" t="s">
-        <v>5354</v>
+        <v>5355</v>
       </c>
       <c r="H1502" s="31"/>
       <c r="I1502" s="32" t="s">
@@ -71339,10 +71342,10 @@
       <c r="A1503" s="29"/>
       <c r="B1503" s="29"/>
       <c r="C1503" s="30" t="s">
-        <v>5355</v>
+        <v>5356</v>
       </c>
       <c r="D1503" s="32" t="s">
-        <v>5321</v>
+        <v>5322</v>
       </c>
       <c r="E1503" s="32" t="s">
         <v>1020</v>
@@ -71351,7 +71354,7 @@
         <v>3850</v>
       </c>
       <c r="G1503" s="32" t="s">
-        <v>5356</v>
+        <v>5357</v>
       </c>
       <c r="H1503" s="31"/>
       <c r="I1503" s="32" t="s">
@@ -71373,10 +71376,10 @@
       <c r="A1504" s="29"/>
       <c r="B1504" s="29"/>
       <c r="C1504" s="30" t="s">
-        <v>5357</v>
+        <v>5358</v>
       </c>
       <c r="D1504" s="32" t="s">
-        <v>5324</v>
+        <v>5325</v>
       </c>
       <c r="E1504" s="32" t="s">
         <v>1020</v>
@@ -71385,7 +71388,7 @@
         <v>3721</v>
       </c>
       <c r="G1504" s="32" t="s">
-        <v>5358</v>
+        <v>5359</v>
       </c>
       <c r="H1504" s="32" t="s">
         <v>1023</v>
@@ -71409,10 +71412,10 @@
       <c r="A1505" s="29"/>
       <c r="B1505" s="29"/>
       <c r="C1505" s="30" t="s">
-        <v>5359</v>
+        <v>5360</v>
       </c>
       <c r="D1505" s="32" t="s">
-        <v>5327</v>
+        <v>5328</v>
       </c>
       <c r="E1505" s="32" t="s">
         <v>1020</v>
@@ -71421,7 +71424,7 @@
         <v>3704</v>
       </c>
       <c r="G1505" s="32" t="s">
-        <v>5360</v>
+        <v>5361</v>
       </c>
       <c r="H1505" s="32" t="s">
         <v>1023</v>
@@ -71445,10 +71448,10 @@
       <c r="A1506" s="29"/>
       <c r="B1506" s="29"/>
       <c r="C1506" s="30" t="s">
-        <v>5361</v>
+        <v>5362</v>
       </c>
       <c r="D1506" s="32" t="s">
-        <v>5330</v>
+        <v>5331</v>
       </c>
       <c r="E1506" s="32" t="s">
         <v>1020</v>
@@ -71457,7 +71460,7 @@
         <v>3683</v>
       </c>
       <c r="G1506" s="32" t="s">
-        <v>5362</v>
+        <v>5363</v>
       </c>
       <c r="H1506" s="32" t="s">
         <v>1023</v>
@@ -71481,10 +71484,10 @@
       <c r="A1507" s="29"/>
       <c r="B1507" s="29"/>
       <c r="C1507" s="30" t="s">
-        <v>5363</v>
+        <v>5364</v>
       </c>
       <c r="D1507" s="32" t="s">
-        <v>5333</v>
+        <v>5334</v>
       </c>
       <c r="E1507" s="32" t="s">
         <v>1020</v>
@@ -71493,7 +71496,7 @@
         <v>3895</v>
       </c>
       <c r="G1507" s="32" t="s">
-        <v>5364</v>
+        <v>5365</v>
       </c>
       <c r="H1507" s="31"/>
       <c r="I1507" s="32" t="s">
@@ -71515,10 +71518,10 @@
       <c r="A1508" s="29"/>
       <c r="B1508" s="29"/>
       <c r="C1508" s="30" t="s">
-        <v>5365</v>
+        <v>5366</v>
       </c>
       <c r="D1508" s="32" t="s">
-        <v>5336</v>
+        <v>5337</v>
       </c>
       <c r="E1508" s="32" t="s">
         <v>1020</v>
@@ -71527,7 +71530,7 @@
         <v>3882</v>
       </c>
       <c r="G1508" s="32" t="s">
-        <v>5366</v>
+        <v>5367</v>
       </c>
       <c r="H1508" s="31"/>
       <c r="I1508" s="32" t="s">
@@ -71549,10 +71552,10 @@
       <c r="A1509" s="29"/>
       <c r="B1509" s="29"/>
       <c r="C1509" s="30" t="s">
-        <v>5367</v>
+        <v>5368</v>
       </c>
       <c r="D1509" s="32" t="s">
-        <v>5339</v>
+        <v>5340</v>
       </c>
       <c r="E1509" s="32" t="s">
         <v>1020</v>
@@ -71561,7 +71564,7 @@
         <v>3866</v>
       </c>
       <c r="G1509" s="32" t="s">
-        <v>5368</v>
+        <v>5369</v>
       </c>
       <c r="H1509" s="31"/>
       <c r="I1509" s="32" t="s">
@@ -71583,10 +71586,10 @@
       <c r="A1510" s="29"/>
       <c r="B1510" s="29"/>
       <c r="C1510" s="30" t="s">
-        <v>5369</v>
+        <v>5370</v>
       </c>
       <c r="D1510" s="32" t="s">
-        <v>5342</v>
+        <v>5343</v>
       </c>
       <c r="E1510" s="32" t="s">
         <v>1020</v>
@@ -71595,7 +71598,7 @@
         <v>3744</v>
       </c>
       <c r="G1510" s="32" t="s">
-        <v>5370</v>
+        <v>5371</v>
       </c>
       <c r="H1510" s="31"/>
       <c r="I1510" s="32" t="s">
@@ -71617,10 +71620,10 @@
       <c r="A1511" s="29"/>
       <c r="B1511" s="29"/>
       <c r="C1511" s="30" t="s">
-        <v>5371</v>
+        <v>5372</v>
       </c>
       <c r="D1511" s="32" t="s">
-        <v>5345</v>
+        <v>5346</v>
       </c>
       <c r="E1511" s="32" t="s">
         <v>1020</v>
@@ -71629,7 +71632,7 @@
         <v>3734</v>
       </c>
       <c r="G1511" s="32" t="s">
-        <v>5372</v>
+        <v>5373</v>
       </c>
       <c r="H1511" s="32" t="s">
         <v>1577</v>
@@ -71653,10 +71656,10 @@
       <c r="A1512" s="29"/>
       <c r="B1512" s="29"/>
       <c r="C1512" s="30" t="s">
-        <v>5373</v>
+        <v>5374</v>
       </c>
       <c r="D1512" s="32" t="s">
-        <v>5374</v>
+        <v>5375</v>
       </c>
       <c r="E1512" s="32" t="s">
         <v>1020</v>
@@ -71665,7 +71668,7 @@
         <v>2605</v>
       </c>
       <c r="G1512" s="32" t="s">
-        <v>5375</v>
+        <v>5376</v>
       </c>
       <c r="H1512" s="31"/>
       <c r="I1512" s="32" t="s">
@@ -71687,10 +71690,10 @@
       <c r="A1513" s="29"/>
       <c r="B1513" s="29"/>
       <c r="C1513" s="30" t="s">
-        <v>5376</v>
+        <v>5377</v>
       </c>
       <c r="D1513" s="32" t="s">
-        <v>5377</v>
+        <v>5378</v>
       </c>
       <c r="E1513" s="32" t="s">
         <v>1020</v>
@@ -71699,7 +71702,7 @@
         <v>2599</v>
       </c>
       <c r="G1513" s="32" t="s">
-        <v>5378</v>
+        <v>5379</v>
       </c>
       <c r="H1513" s="31"/>
       <c r="I1513" s="32" t="s">
@@ -71721,10 +71724,10 @@
       <c r="A1514" s="29"/>
       <c r="B1514" s="29"/>
       <c r="C1514" s="30" t="s">
-        <v>5379</v>
+        <v>5380</v>
       </c>
       <c r="D1514" s="32" t="s">
-        <v>5380</v>
+        <v>5381</v>
       </c>
       <c r="E1514" s="32" t="s">
         <v>3328</v>
@@ -71733,7 +71736,7 @@
         <v>3329</v>
       </c>
       <c r="G1514" s="32" t="s">
-        <v>5381</v>
+        <v>5382</v>
       </c>
       <c r="H1514" s="31"/>
       <c r="I1514" s="32" t="s">
@@ -71755,10 +71758,10 @@
       <c r="A1515" s="29"/>
       <c r="B1515" s="29"/>
       <c r="C1515" s="30" t="s">
-        <v>5382</v>
+        <v>5383</v>
       </c>
       <c r="D1515" s="32" t="s">
-        <v>5383</v>
+        <v>5384</v>
       </c>
       <c r="E1515" s="32" t="s">
         <v>2831</v>
@@ -71767,7 +71770,7 @@
         <v>2832</v>
       </c>
       <c r="G1515" s="32" t="s">
-        <v>5384</v>
+        <v>5385</v>
       </c>
       <c r="H1515" s="31"/>
       <c r="I1515" s="32" t="s">
@@ -71789,10 +71792,10 @@
       <c r="A1516" s="29"/>
       <c r="B1516" s="29"/>
       <c r="C1516" s="30" t="s">
-        <v>5385</v>
+        <v>5386</v>
       </c>
       <c r="D1516" s="32" t="s">
-        <v>5386</v>
+        <v>5387</v>
       </c>
       <c r="E1516" s="32" t="s">
         <v>3058</v>
@@ -71801,7 +71804,7 @@
         <v>3059</v>
       </c>
       <c r="G1516" s="32" t="s">
-        <v>5387</v>
+        <v>5388</v>
       </c>
       <c r="H1516" s="31"/>
       <c r="I1516" s="32" t="s">
@@ -71823,10 +71826,10 @@
       <c r="A1517" s="29"/>
       <c r="B1517" s="29"/>
       <c r="C1517" s="30" t="s">
-        <v>5388</v>
+        <v>5389</v>
       </c>
       <c r="D1517" s="32" t="s">
-        <v>5389</v>
+        <v>5390</v>
       </c>
       <c r="E1517" s="32" t="s">
         <v>2632</v>
@@ -71835,7 +71838,7 @@
         <v>2613</v>
       </c>
       <c r="G1517" s="32" t="s">
-        <v>5390</v>
+        <v>5391</v>
       </c>
       <c r="H1517" s="31"/>
       <c r="I1517" s="32" t="s">
@@ -71857,10 +71860,10 @@
       <c r="A1518" s="29"/>
       <c r="B1518" s="29"/>
       <c r="C1518" s="30" t="s">
-        <v>5391</v>
+        <v>5392</v>
       </c>
       <c r="D1518" s="32" t="s">
-        <v>5392</v>
+        <v>5393</v>
       </c>
       <c r="E1518" s="32" t="s">
         <v>3050</v>
@@ -71869,7 +71872,7 @@
         <v>3051</v>
       </c>
       <c r="G1518" s="32" t="s">
-        <v>5393</v>
+        <v>5394</v>
       </c>
       <c r="H1518" s="31"/>
       <c r="I1518" s="32" t="s">
@@ -71891,17 +71894,17 @@
       <c r="A1519" s="29"/>
       <c r="B1519" s="29"/>
       <c r="C1519" s="30" t="s">
-        <v>5394</v>
+        <v>5395</v>
       </c>
       <c r="D1519" s="32" t="s">
-        <v>5395</v>
+        <v>5396</v>
       </c>
       <c r="E1519" s="32" t="s">
         <v>2734</v>
       </c>
       <c r="F1519" s="32"/>
       <c r="G1519" s="32" t="s">
-        <v>5396</v>
+        <v>5397</v>
       </c>
       <c r="H1519" s="31"/>
       <c r="I1519" s="32"/>
@@ -71919,17 +71922,17 @@
       <c r="A1520" s="29"/>
       <c r="B1520" s="29"/>
       <c r="C1520" s="30" t="s">
-        <v>5397</v>
+        <v>5398</v>
       </c>
       <c r="D1520" s="32" t="s">
-        <v>5398</v>
+        <v>5399</v>
       </c>
       <c r="E1520" s="32" t="s">
         <v>2997</v>
       </c>
       <c r="F1520" s="32"/>
       <c r="G1520" s="32" t="s">
-        <v>5399</v>
+        <v>5400</v>
       </c>
       <c r="H1520" s="31"/>
       <c r="I1520" s="32"/>
@@ -71992,13 +71995,13 @@
         <v>34</v>
       </c>
       <c r="D1" s="24" t="s">
-        <v>5400</v>
+        <v>5401</v>
       </c>
       <c r="E1" s="25" t="s">
-        <v>5401</v>
+        <v>5402</v>
       </c>
       <c r="F1" s="25" t="s">
-        <v>5402</v>
+        <v>5403</v>
       </c>
       <c r="G1" s="22"/>
       <c r="H1" s="22"/>
@@ -72010,7 +72013,7 @@
         <v>3776</v>
       </c>
       <c r="D2" s="35" t="s">
-        <v>5403</v>
+        <v>5404</v>
       </c>
       <c r="E2" s="35" t="s">
         <v>3770</v>
@@ -72026,7 +72029,7 @@
         <v>3776</v>
       </c>
       <c r="D3" s="35" t="s">
-        <v>5403</v>
+        <v>5404</v>
       </c>
       <c r="E3" s="35" t="s">
         <v>3673</v>
@@ -72042,7 +72045,7 @@
         <v>3776</v>
       </c>
       <c r="D4" s="35" t="s">
-        <v>5403</v>
+        <v>5404</v>
       </c>
       <c r="E4" s="35" t="s">
         <v>3783</v>
@@ -72060,7 +72063,7 @@
         <v>3776</v>
       </c>
       <c r="D5" s="35" t="s">
-        <v>5403</v>
+        <v>5404</v>
       </c>
       <c r="E5" s="35" t="s">
         <v>3788</v>
@@ -72078,7 +72081,7 @@
         <v>3776</v>
       </c>
       <c r="D6" s="35" t="s">
-        <v>5403</v>
+        <v>5404</v>
       </c>
       <c r="E6" s="35" t="s">
         <v>3675</v>
@@ -72094,7 +72097,7 @@
         <v>1659</v>
       </c>
       <c r="D7" s="35" t="s">
-        <v>5403</v>
+        <v>5404</v>
       </c>
       <c r="E7" s="35" t="s">
         <v>1654</v>
@@ -72110,7 +72113,7 @@
         <v>1659</v>
       </c>
       <c r="D8" s="35" t="s">
-        <v>5403</v>
+        <v>5404</v>
       </c>
       <c r="E8" s="35" t="s">
         <v>919</v>
@@ -72126,7 +72129,7 @@
         <v>1659</v>
       </c>
       <c r="D9" s="35" t="s">
-        <v>5403</v>
+        <v>5404</v>
       </c>
       <c r="E9" s="35" t="s">
         <v>1761</v>
@@ -72146,7 +72149,7 @@
         <v>1659</v>
       </c>
       <c r="D10" s="35" t="s">
-        <v>5403</v>
+        <v>5404</v>
       </c>
       <c r="E10" s="35" t="s">
         <v>1761</v>
@@ -72166,7 +72169,7 @@
         <v>1659</v>
       </c>
       <c r="D11" s="35" t="s">
-        <v>5403</v>
+        <v>5404</v>
       </c>
       <c r="E11" s="35" t="s">
         <v>1761</v>
@@ -72186,7 +72189,7 @@
         <v>1659</v>
       </c>
       <c r="D12" s="35" t="s">
-        <v>5403</v>
+        <v>5404</v>
       </c>
       <c r="E12" s="35" t="s">
         <v>1777</v>
@@ -72206,7 +72209,7 @@
         <v>1659</v>
       </c>
       <c r="D13" s="35" t="s">
-        <v>5403</v>
+        <v>5404</v>
       </c>
       <c r="E13" s="35" t="s">
         <v>1797</v>
@@ -72224,7 +72227,7 @@
         <v>3795</v>
       </c>
       <c r="D14" s="35" t="s">
-        <v>5403</v>
+        <v>5404</v>
       </c>
       <c r="E14" s="35" t="s">
         <v>3783</v>
@@ -72242,7 +72245,7 @@
         <v>3795</v>
       </c>
       <c r="D15" s="35" t="s">
-        <v>5403</v>
+        <v>5404</v>
       </c>
       <c r="E15" s="35" t="s">
         <v>3783</v>
@@ -72255,10 +72258,10 @@
       <c r="A16" s="33"/>
       <c r="B16" s="33"/>
       <c r="C16" s="34" t="s">
-        <v>5404</v>
+        <v>5405</v>
       </c>
       <c r="D16" s="35" t="s">
-        <v>5405</v>
+        <v>5406</v>
       </c>
       <c r="E16" s="35" t="s">
         <v>2117</v>
@@ -72274,7 +72277,7 @@
         <v>2275</v>
       </c>
       <c r="D17" s="35" t="s">
-        <v>5405</v>
+        <v>5406</v>
       </c>
       <c r="E17" s="35" t="s">
         <v>2117</v>
@@ -72290,7 +72293,7 @@
         <v>2279</v>
       </c>
       <c r="D18" s="35" t="s">
-        <v>5405</v>
+        <v>5406</v>
       </c>
       <c r="E18" s="35" t="s">
         <v>2117</v>
@@ -72306,7 +72309,7 @@
         <v>2305</v>
       </c>
       <c r="D19" s="35" t="s">
-        <v>5406</v>
+        <v>5407</v>
       </c>
       <c r="E19" s="35" t="s">
         <v>2299</v>
@@ -72322,7 +72325,7 @@
         <v>427</v>
       </c>
       <c r="D20" s="35" t="s">
-        <v>5406</v>
+        <v>5407</v>
       </c>
       <c r="E20" s="35" t="s">
         <v>418</v>
@@ -72342,7 +72345,7 @@
         <v>776</v>
       </c>
       <c r="D21" s="35" t="s">
-        <v>5406</v>
+        <v>5407</v>
       </c>
       <c r="E21" s="35" t="s">
         <v>770</v>
@@ -72358,7 +72361,7 @@
         <v>3606</v>
       </c>
       <c r="D22" s="35" t="s">
-        <v>5406</v>
+        <v>5407</v>
       </c>
       <c r="E22" s="35" t="s">
         <v>3603</v>
@@ -72374,7 +72377,7 @@
         <v>2153</v>
       </c>
       <c r="D23" s="35" t="s">
-        <v>5406</v>
+        <v>5407</v>
       </c>
       <c r="E23" s="35" t="s">
         <v>2152</v>
@@ -72390,7 +72393,7 @@
         <v>3381</v>
       </c>
       <c r="D24" s="35" t="s">
-        <v>5406</v>
+        <v>5407</v>
       </c>
       <c r="E24" s="35" t="s">
         <v>3380</v>
@@ -72406,7 +72409,7 @@
         <v>1818</v>
       </c>
       <c r="D25" s="35" t="s">
-        <v>5407</v>
+        <v>5408</v>
       </c>
       <c r="E25" s="35" t="s">
         <v>625</v>
@@ -72422,7 +72425,7 @@
         <v>1818</v>
       </c>
       <c r="D26" s="35" t="s">
-        <v>5407</v>
+        <v>5408</v>
       </c>
       <c r="E26" s="35" t="s">
         <v>1610</v>
@@ -72438,7 +72441,7 @@
         <v>3830</v>
       </c>
       <c r="D27" s="35" t="s">
-        <v>5407</v>
+        <v>5408</v>
       </c>
       <c r="E27" s="35" t="s">
         <v>3538</v>
@@ -72454,7 +72457,7 @@
         <v>3830</v>
       </c>
       <c r="D28" s="35" t="s">
-        <v>5407</v>
+        <v>5408</v>
       </c>
       <c r="E28" s="35" t="s">
         <v>3827</v>
@@ -72470,7 +72473,7 @@
         <v>4014</v>
       </c>
       <c r="D29" s="35" t="s">
-        <v>5408</v>
+        <v>5409</v>
       </c>
       <c r="E29" s="35" t="s">
         <v>4005</v>
@@ -72488,7 +72491,7 @@
         <v>4014</v>
       </c>
       <c r="D30" s="35" t="s">
-        <v>5408</v>
+        <v>5409</v>
       </c>
       <c r="E30" s="35" t="s">
         <v>4005</v>
@@ -72504,7 +72507,7 @@
         <v>4006</v>
       </c>
       <c r="D31" s="35" t="s">
-        <v>5408</v>
+        <v>5409</v>
       </c>
       <c r="E31" s="35" t="s">
         <v>4005</v>
@@ -72721,10 +72724,10 @@
       <c r="A44" s="33"/>
       <c r="B44" s="33"/>
       <c r="C44" s="34" t="s">
-        <v>5409</v>
+        <v>5410</v>
       </c>
       <c r="D44" s="35" t="s">
-        <v>5410</v>
+        <v>5411</v>
       </c>
       <c r="E44" s="35" t="s">
         <v>2117</v>
@@ -72740,7 +72743,7 @@
         <v>2261</v>
       </c>
       <c r="D45" s="35" t="s">
-        <v>5410</v>
+        <v>5411</v>
       </c>
       <c r="E45" s="35" t="s">
         <v>2117</v>
@@ -72756,7 +72759,7 @@
         <v>2265</v>
       </c>
       <c r="D46" s="35" t="s">
-        <v>5410</v>
+        <v>5411</v>
       </c>
       <c r="E46" s="35" t="s">
         <v>2117</v>
@@ -72771,10 +72774,10 @@
         <v>282</v>
       </c>
       <c r="C47" s="34" t="s">
-        <v>5411</v>
+        <v>5412</v>
       </c>
       <c r="D47" s="35" t="s">
-        <v>5412</v>
+        <v>5413</v>
       </c>
       <c r="E47" s="35" t="s">
         <v>2966</v>
@@ -72790,7 +72793,7 @@
         <v>3338</v>
       </c>
       <c r="D48" s="35" t="s">
-        <v>5413</v>
+        <v>5414</v>
       </c>
       <c r="E48" s="35" t="s">
         <v>2117</v>
@@ -72808,7 +72811,7 @@
         <v>3338</v>
       </c>
       <c r="D49" s="35" t="s">
-        <v>5413</v>
+        <v>5414</v>
       </c>
       <c r="E49" s="35" t="s">
         <v>2117</v>
@@ -72826,7 +72829,7 @@
         <v>3338</v>
       </c>
       <c r="D50" s="35" t="s">
-        <v>5413</v>
+        <v>5414</v>
       </c>
       <c r="E50" s="35" t="s">
         <v>3333</v>
@@ -72889,7 +72892,7 @@
         <v>282</v>
       </c>
       <c r="C54" s="34" t="s">
-        <v>5414</v>
+        <v>5415</v>
       </c>
       <c r="D54" s="35" t="s">
         <v>201</v>
@@ -72909,10 +72912,10 @@
         <v>282</v>
       </c>
       <c r="C55" s="34" t="s">
-        <v>5415</v>
+        <v>5416</v>
       </c>
       <c r="D55" s="35" t="s">
-        <v>5416</v>
+        <v>5417</v>
       </c>
       <c r="E55" s="35" t="s">
         <v>1354</v>
@@ -72932,7 +72935,7 @@
         <v>1363</v>
       </c>
       <c r="D56" s="35" t="s">
-        <v>5416</v>
+        <v>5417</v>
       </c>
       <c r="E56" s="35" t="s">
         <v>1354</v>
@@ -72948,13 +72951,13 @@
         <v>2075</v>
       </c>
       <c r="D57" s="35" t="s">
-        <v>5417</v>
+        <v>5418</v>
       </c>
       <c r="E57" s="35" t="s">
-        <v>5418</v>
+        <v>5419</v>
       </c>
       <c r="F57" s="34" t="s">
-        <v>5419</v>
+        <v>5420</v>
       </c>
     </row>
     <row r="58">
@@ -72964,7 +72967,7 @@
         <v>2075</v>
       </c>
       <c r="D58" s="35" t="s">
-        <v>5417</v>
+        <v>5418</v>
       </c>
       <c r="E58" s="35" t="s">
         <v>2086</v>
@@ -72984,7 +72987,7 @@
         <v>2075</v>
       </c>
       <c r="D59" s="35" t="s">
-        <v>5417</v>
+        <v>5418</v>
       </c>
       <c r="E59" s="35" t="s">
         <v>2086</v>
@@ -73000,7 +73003,7 @@
         <v>2075</v>
       </c>
       <c r="D60" s="35" t="s">
-        <v>5417</v>
+        <v>5418</v>
       </c>
       <c r="E60" s="35" t="s">
         <v>2067</v>
@@ -73016,7 +73019,7 @@
         <v>2174</v>
       </c>
       <c r="D61" s="35" t="s">
-        <v>5420</v>
+        <v>5421</v>
       </c>
       <c r="E61" s="35" t="s">
         <v>2119</v>
@@ -73032,7 +73035,7 @@
         <v>2317</v>
       </c>
       <c r="D62" s="35" t="s">
-        <v>5420</v>
+        <v>5421</v>
       </c>
       <c r="E62" s="35" t="s">
         <v>2282</v>
@@ -73120,7 +73123,7 @@
         <v>48</v>
       </c>
       <c r="D67" s="35" t="s">
-        <v>5421</v>
+        <v>5422</v>
       </c>
       <c r="E67" s="35" t="s">
         <v>1205</v>
@@ -73133,10 +73136,10 @@
       <c r="A68" s="33"/>
       <c r="B68" s="33"/>
       <c r="C68" s="34" t="s">
-        <v>5422</v>
+        <v>5423</v>
       </c>
       <c r="D68" s="35" t="s">
-        <v>5423</v>
+        <v>5424</v>
       </c>
       <c r="E68" s="35" t="s">
         <v>2495</v>
@@ -73152,7 +73155,7 @@
         <v>3500</v>
       </c>
       <c r="D69" s="35" t="s">
-        <v>5424</v>
+        <v>5425</v>
       </c>
       <c r="E69" s="35" t="s">
         <v>3499</v>
@@ -73168,7 +73171,7 @@
         <v>3446</v>
       </c>
       <c r="D70" s="35" t="s">
-        <v>5424</v>
+        <v>5425</v>
       </c>
       <c r="E70" s="35" t="s">
         <v>3445</v>
@@ -73184,7 +73187,7 @@
         <v>3446</v>
       </c>
       <c r="D71" s="35" t="s">
-        <v>5424</v>
+        <v>5425</v>
       </c>
       <c r="E71" s="35" t="s">
         <v>3459</v>
@@ -73200,7 +73203,7 @@
         <v>3446</v>
       </c>
       <c r="D72" s="35" t="s">
-        <v>5424</v>
+        <v>5425</v>
       </c>
       <c r="E72" s="35" t="s">
         <v>3480</v>
@@ -73216,7 +73219,7 @@
         <v>3446</v>
       </c>
       <c r="D73" s="35" t="s">
-        <v>5424</v>
+        <v>5425</v>
       </c>
       <c r="E73" s="35" t="s">
         <v>3499</v>
@@ -73236,7 +73239,7 @@
         <v>1262</v>
       </c>
       <c r="D74" s="35" t="s">
-        <v>5425</v>
+        <v>5426</v>
       </c>
       <c r="E74" s="35" t="s">
         <v>1236</v>
@@ -73256,7 +73259,7 @@
         <v>2055</v>
       </c>
       <c r="D75" s="35" t="s">
-        <v>5425</v>
+        <v>5426</v>
       </c>
       <c r="E75" s="35" t="s">
         <v>2042</v>
@@ -73276,7 +73279,7 @@
         <v>1166</v>
       </c>
       <c r="D76" s="35" t="s">
-        <v>5425</v>
+        <v>5426</v>
       </c>
       <c r="E76" s="35" t="s">
         <v>1155</v>
@@ -73292,7 +73295,7 @@
         <v>2311</v>
       </c>
       <c r="D77" s="35" t="s">
-        <v>5426</v>
+        <v>5427</v>
       </c>
       <c r="E77" s="35" t="s">
         <v>2282</v>
@@ -73308,7 +73311,7 @@
         <v>2311</v>
       </c>
       <c r="D78" s="35" t="s">
-        <v>5426</v>
+        <v>5427</v>
       </c>
       <c r="E78" s="35" t="s">
         <v>2342</v>
@@ -73324,7 +73327,7 @@
         <v>2311</v>
       </c>
       <c r="D79" s="35" t="s">
-        <v>5426</v>
+        <v>5427</v>
       </c>
       <c r="E79" s="35" t="s">
         <v>2299</v>
@@ -73340,7 +73343,7 @@
         <v>3724</v>
       </c>
       <c r="D80" s="35" t="s">
-        <v>5426</v>
+        <v>5427</v>
       </c>
       <c r="E80" s="35" t="s">
         <v>3715</v>
@@ -73356,7 +73359,7 @@
         <v>1096</v>
       </c>
       <c r="D81" s="35" t="s">
-        <v>5426</v>
+        <v>5427</v>
       </c>
       <c r="E81" s="35" t="s">
         <v>1080</v>
@@ -73372,7 +73375,7 @@
         <v>3707</v>
       </c>
       <c r="D82" s="35" t="s">
-        <v>5426</v>
+        <v>5427</v>
       </c>
       <c r="E82" s="35" t="s">
         <v>3698</v>
@@ -73388,7 +73391,7 @@
         <v>1064</v>
       </c>
       <c r="D83" s="35" t="s">
-        <v>5426</v>
+        <v>5427</v>
       </c>
       <c r="E83" s="35" t="s">
         <v>1048</v>
@@ -73404,7 +73407,7 @@
         <v>3901</v>
       </c>
       <c r="D84" s="35" t="s">
-        <v>5426</v>
+        <v>5427</v>
       </c>
       <c r="E84" s="35" t="s">
         <v>3863</v>
@@ -73420,7 +73423,7 @@
         <v>1946</v>
       </c>
       <c r="D85" s="35" t="s">
-        <v>5426</v>
+        <v>5427</v>
       </c>
       <c r="E85" s="35" t="s">
         <v>1874</v>
@@ -73436,7 +73439,7 @@
         <v>3859</v>
       </c>
       <c r="D86" s="35" t="s">
-        <v>5426</v>
+        <v>5427</v>
       </c>
       <c r="E86" s="35" t="s">
         <v>3673</v>
@@ -73452,7 +73455,7 @@
         <v>1867</v>
       </c>
       <c r="D87" s="35" t="s">
-        <v>5426</v>
+        <v>5427</v>
       </c>
       <c r="E87" s="35" t="s">
         <v>919</v>
@@ -73468,7 +73471,7 @@
         <v>3845</v>
       </c>
       <c r="D88" s="35" t="s">
-        <v>5426</v>
+        <v>5427</v>
       </c>
       <c r="E88" s="35" t="s">
         <v>3673</v>
@@ -73484,7 +73487,7 @@
         <v>1844</v>
       </c>
       <c r="D89" s="35" t="s">
-        <v>5426</v>
+        <v>5427</v>
       </c>
       <c r="E89" s="35" t="s">
         <v>919</v>
@@ -73500,7 +73503,7 @@
         <v>1900</v>
       </c>
       <c r="D90" s="35" t="s">
-        <v>5426</v>
+        <v>5427</v>
       </c>
       <c r="E90" s="35" t="s">
         <v>1874</v>
@@ -73516,7 +73519,7 @@
         <v>3877</v>
       </c>
       <c r="D91" s="35" t="s">
-        <v>5426</v>
+        <v>5427</v>
       </c>
       <c r="E91" s="35" t="s">
         <v>3863</v>
@@ -73532,7 +73535,7 @@
         <v>3891</v>
       </c>
       <c r="D92" s="35" t="s">
-        <v>5426</v>
+        <v>5427</v>
       </c>
       <c r="E92" s="35" t="s">
         <v>3863</v>
@@ -73548,7 +73551,7 @@
         <v>1923</v>
       </c>
       <c r="D93" s="35" t="s">
-        <v>5426</v>
+        <v>5427</v>
       </c>
       <c r="E93" s="35" t="s">
         <v>1874</v>
@@ -73564,7 +73567,7 @@
         <v>3687</v>
       </c>
       <c r="D94" s="35" t="s">
-        <v>5426</v>
+        <v>5427</v>
       </c>
       <c r="E94" s="35" t="s">
         <v>3677</v>
@@ -73580,7 +73583,7 @@
         <v>1027</v>
       </c>
       <c r="D95" s="35" t="s">
-        <v>5426</v>
+        <v>5427</v>
       </c>
       <c r="E95" s="35" t="s">
         <v>1005</v>
@@ -73596,7 +73599,7 @@
         <v>3750</v>
       </c>
       <c r="D96" s="35" t="s">
-        <v>5426</v>
+        <v>5427</v>
       </c>
       <c r="E96" s="35" t="s">
         <v>3673</v>
@@ -73612,7 +73615,7 @@
         <v>1603</v>
       </c>
       <c r="D97" s="35" t="s">
-        <v>5426</v>
+        <v>5427</v>
       </c>
       <c r="E97" s="35" t="s">
         <v>919</v>
@@ -73628,7 +73631,7 @@
         <v>3739</v>
       </c>
       <c r="D98" s="35" t="s">
-        <v>5426</v>
+        <v>5427</v>
       </c>
       <c r="E98" s="35" t="s">
         <v>3673</v>
@@ -73644,7 +73647,7 @@
         <v>1580</v>
       </c>
       <c r="D99" s="35" t="s">
-        <v>5426</v>
+        <v>5427</v>
       </c>
       <c r="E99" s="35" t="s">
         <v>1557</v>
@@ -73660,7 +73663,7 @@
         <v>2167</v>
       </c>
       <c r="D100" s="35" t="s">
-        <v>5426</v>
+        <v>5427</v>
       </c>
       <c r="E100" s="35" t="s">
         <v>2119</v>
@@ -73676,7 +73679,7 @@
         <v>2167</v>
       </c>
       <c r="D101" s="35" t="s">
-        <v>5426</v>
+        <v>5427</v>
       </c>
       <c r="E101" s="35" t="s">
         <v>2215</v>
@@ -73692,7 +73695,7 @@
         <v>2300</v>
       </c>
       <c r="D102" s="35" t="s">
-        <v>5426</v>
+        <v>5427</v>
       </c>
       <c r="E102" s="35" t="s">
         <v>2299</v>
@@ -73843,10 +73846,10 @@
         <v>1207</v>
       </c>
       <c r="C111" s="34" t="s">
-        <v>5427</v>
+        <v>5428</v>
       </c>
       <c r="D111" s="35" t="s">
-        <v>5428</v>
+        <v>5429</v>
       </c>
       <c r="E111" s="35" t="s">
         <v>3936</v>
@@ -73862,7 +73865,7 @@
         <v>3905</v>
       </c>
       <c r="D112" s="35" t="s">
-        <v>5428</v>
+        <v>5429</v>
       </c>
       <c r="E112" s="35" t="s">
         <v>3904</v>
@@ -73878,7 +73881,7 @@
         <v>3916</v>
       </c>
       <c r="D113" s="35" t="s">
-        <v>5428</v>
+        <v>5429</v>
       </c>
       <c r="E113" s="35" t="s">
         <v>3938</v>
@@ -73894,7 +73897,7 @@
         <v>3916</v>
       </c>
       <c r="D114" s="35" t="s">
-        <v>5428</v>
+        <v>5429</v>
       </c>
       <c r="E114" s="35" t="s">
         <v>3915</v>
@@ -73910,7 +73913,7 @@
         <v>3924</v>
       </c>
       <c r="D115" s="35" t="s">
-        <v>5429</v>
+        <v>5430</v>
       </c>
       <c r="E115" s="35" t="s">
         <v>3936</v>
@@ -73928,7 +73931,7 @@
         <v>3924</v>
       </c>
       <c r="D116" s="35" t="s">
-        <v>5429</v>
+        <v>5430</v>
       </c>
       <c r="E116" s="35" t="s">
         <v>3936</v>
@@ -73944,7 +73947,7 @@
         <v>3924</v>
       </c>
       <c r="D117" s="35" t="s">
-        <v>5429</v>
+        <v>5430</v>
       </c>
       <c r="E117" s="35" t="s">
         <v>3938</v>
@@ -73960,7 +73963,7 @@
         <v>3924</v>
       </c>
       <c r="D118" s="35" t="s">
-        <v>5429</v>
+        <v>5430</v>
       </c>
       <c r="E118" s="35" t="s">
         <v>3915</v>
@@ -74041,10 +74044,10 @@
         <v>282</v>
       </c>
       <c r="C123" s="34" t="s">
-        <v>5430</v>
+        <v>5431</v>
       </c>
       <c r="D123" s="35" t="s">
-        <v>5431</v>
+        <v>5432</v>
       </c>
       <c r="E123" s="35" t="s">
         <v>2584</v>
@@ -74060,7 +74063,7 @@
         <v>476</v>
       </c>
       <c r="D124" s="35" t="s">
-        <v>5432</v>
+        <v>5433</v>
       </c>
       <c r="E124" s="35" t="s">
         <v>413</v>
@@ -74076,7 +74079,7 @@
         <v>476</v>
       </c>
       <c r="D125" s="35" t="s">
-        <v>5432</v>
+        <v>5433</v>
       </c>
       <c r="E125" s="35" t="s">
         <v>418</v>
@@ -74092,7 +74095,7 @@
         <v>476</v>
       </c>
       <c r="D126" s="35" t="s">
-        <v>5432</v>
+        <v>5433</v>
       </c>
       <c r="E126" s="35" t="s">
         <v>4068</v>
@@ -74108,7 +74111,7 @@
         <v>476</v>
       </c>
       <c r="D127" s="35" t="s">
-        <v>5432</v>
+        <v>5433</v>
       </c>
       <c r="E127" s="35" t="s">
         <v>4037</v>
@@ -74124,7 +74127,7 @@
         <v>476</v>
       </c>
       <c r="D128" s="35" t="s">
-        <v>5432</v>
+        <v>5433</v>
       </c>
       <c r="E128" s="35" t="s">
         <v>4047</v>
@@ -74140,7 +74143,7 @@
         <v>476</v>
       </c>
       <c r="D129" s="35" t="s">
-        <v>5432</v>
+        <v>5433</v>
       </c>
       <c r="E129" s="35" t="s">
         <v>4005</v>
@@ -74156,7 +74159,7 @@
         <v>3975</v>
       </c>
       <c r="D130" s="35" t="s">
-        <v>5432</v>
+        <v>5433</v>
       </c>
       <c r="E130" s="35" t="s">
         <v>3974</v>
@@ -74172,7 +74175,7 @@
         <v>658</v>
       </c>
       <c r="D131" s="35" t="s">
-        <v>5432</v>
+        <v>5433</v>
       </c>
       <c r="E131" s="35" t="s">
         <v>647</v>
@@ -74192,7 +74195,7 @@
         <v>658</v>
       </c>
       <c r="D132" s="35" t="s">
-        <v>5432</v>
+        <v>5433</v>
       </c>
       <c r="E132" s="35" t="s">
         <v>647</v>
@@ -74208,7 +74211,7 @@
         <v>658</v>
       </c>
       <c r="D133" s="35" t="s">
-        <v>5432</v>
+        <v>5433</v>
       </c>
       <c r="E133" s="35" t="s">
         <v>874</v>
@@ -74228,7 +74231,7 @@
         <v>658</v>
       </c>
       <c r="D134" s="35" t="s">
-        <v>5432</v>
+        <v>5433</v>
       </c>
       <c r="E134" s="35" t="s">
         <v>874</v>
@@ -74248,7 +74251,7 @@
         <v>658</v>
       </c>
       <c r="D135" s="35" t="s">
-        <v>5432</v>
+        <v>5433</v>
       </c>
       <c r="E135" s="35" t="s">
         <v>874</v>
@@ -74264,7 +74267,7 @@
         <v>658</v>
       </c>
       <c r="D136" s="35" t="s">
-        <v>5432</v>
+        <v>5433</v>
       </c>
       <c r="E136" s="35" t="s">
         <v>815</v>
@@ -74284,7 +74287,7 @@
         <v>658</v>
       </c>
       <c r="D137" s="35" t="s">
-        <v>5432</v>
+        <v>5433</v>
       </c>
       <c r="E137" s="35" t="s">
         <v>815</v>
@@ -74300,7 +74303,7 @@
         <v>658</v>
       </c>
       <c r="D138" s="35" t="s">
-        <v>5432</v>
+        <v>5433</v>
       </c>
       <c r="E138" s="35" t="s">
         <v>770</v>
@@ -74320,7 +74323,7 @@
         <v>658</v>
       </c>
       <c r="D139" s="35" t="s">
-        <v>5432</v>
+        <v>5433</v>
       </c>
       <c r="E139" s="35" t="s">
         <v>770</v>
@@ -74336,7 +74339,7 @@
         <v>658</v>
       </c>
       <c r="D140" s="35" t="s">
-        <v>5432</v>
+        <v>5433</v>
       </c>
       <c r="E140" s="35" t="s">
         <v>919</v>
@@ -74356,7 +74359,7 @@
         <v>658</v>
       </c>
       <c r="D141" s="35" t="s">
-        <v>5432</v>
+        <v>5433</v>
       </c>
       <c r="E141" s="35" t="s">
         <v>919</v>
@@ -74372,7 +74375,7 @@
         <v>658</v>
       </c>
       <c r="D142" s="35" t="s">
-        <v>5432</v>
+        <v>5433</v>
       </c>
       <c r="E142" s="35" t="s">
         <v>1436</v>
@@ -74388,7 +74391,7 @@
         <v>658</v>
       </c>
       <c r="D143" s="35" t="s">
-        <v>5432</v>
+        <v>5433</v>
       </c>
       <c r="E143" s="35" t="s">
         <v>1550</v>
@@ -74408,7 +74411,7 @@
         <v>658</v>
       </c>
       <c r="D144" s="35" t="s">
-        <v>5432</v>
+        <v>5433</v>
       </c>
       <c r="E144" s="35" t="s">
         <v>1499</v>
@@ -74424,7 +74427,7 @@
         <v>658</v>
       </c>
       <c r="D145" s="35" t="s">
-        <v>5432</v>
+        <v>5433</v>
       </c>
       <c r="E145" s="35" t="s">
         <v>1291</v>
@@ -74440,7 +74443,7 @@
         <v>364</v>
       </c>
       <c r="D146" s="35" t="s">
-        <v>5432</v>
+        <v>5433</v>
       </c>
       <c r="E146" s="35" t="s">
         <v>331</v>
@@ -74460,7 +74463,7 @@
         <v>364</v>
       </c>
       <c r="D147" s="35" t="s">
-        <v>5432</v>
+        <v>5433</v>
       </c>
       <c r="E147" s="35" t="s">
         <v>331</v>
@@ -74476,7 +74479,7 @@
         <v>364</v>
       </c>
       <c r="D148" s="35" t="s">
-        <v>5432</v>
+        <v>5433</v>
       </c>
       <c r="E148" s="35" t="s">
         <v>413</v>
@@ -74492,7 +74495,7 @@
         <v>3562</v>
       </c>
       <c r="D149" s="35" t="s">
-        <v>5432</v>
+        <v>5433</v>
       </c>
       <c r="E149" s="35" t="s">
         <v>3550</v>
@@ -74508,7 +74511,7 @@
         <v>3562</v>
       </c>
       <c r="D150" s="35" t="s">
-        <v>5432</v>
+        <v>5433</v>
       </c>
       <c r="E150" s="35" t="s">
         <v>3633</v>
@@ -74526,7 +74529,7 @@
         <v>3562</v>
       </c>
       <c r="D151" s="35" t="s">
-        <v>5432</v>
+        <v>5433</v>
       </c>
       <c r="E151" s="35" t="s">
         <v>3659</v>
@@ -74542,7 +74545,7 @@
         <v>3562</v>
       </c>
       <c r="D152" s="35" t="s">
-        <v>5432</v>
+        <v>5433</v>
       </c>
       <c r="E152" s="35" t="s">
         <v>3601</v>
@@ -74558,7 +74561,7 @@
         <v>3562</v>
       </c>
       <c r="D153" s="35" t="s">
-        <v>5432</v>
+        <v>5433</v>
       </c>
       <c r="E153" s="35" t="s">
         <v>3603</v>
@@ -74576,7 +74579,7 @@
         <v>3562</v>
       </c>
       <c r="D154" s="35" t="s">
-        <v>5432</v>
+        <v>5433</v>
       </c>
       <c r="E154" s="35" t="s">
         <v>3673</v>
@@ -74592,7 +74595,7 @@
         <v>359</v>
       </c>
       <c r="D155" s="35" t="s">
-        <v>5432</v>
+        <v>5433</v>
       </c>
       <c r="E155" s="35" t="s">
         <v>331</v>
@@ -74612,7 +74615,7 @@
         <v>359</v>
       </c>
       <c r="D156" s="35" t="s">
-        <v>5432</v>
+        <v>5433</v>
       </c>
       <c r="E156" s="35" t="s">
         <v>331</v>
@@ -74628,7 +74631,7 @@
         <v>359</v>
       </c>
       <c r="D157" s="35" t="s">
-        <v>5432</v>
+        <v>5433</v>
       </c>
       <c r="E157" s="35" t="s">
         <v>413</v>
@@ -74644,7 +74647,7 @@
         <v>3962</v>
       </c>
       <c r="D158" s="35" t="s">
-        <v>5432</v>
+        <v>5433</v>
       </c>
       <c r="E158" s="35" t="s">
         <v>3974</v>
@@ -74662,7 +74665,7 @@
         <v>3962</v>
       </c>
       <c r="D159" s="35" t="s">
-        <v>5432</v>
+        <v>5433</v>
       </c>
       <c r="E159" s="35" t="s">
         <v>1422</v>
@@ -74678,7 +74681,7 @@
         <v>3962</v>
       </c>
       <c r="D160" s="35" t="s">
-        <v>5432</v>
+        <v>5433</v>
       </c>
       <c r="E160" s="35" t="s">
         <v>2726</v>
@@ -74694,7 +74697,7 @@
         <v>3962</v>
       </c>
       <c r="D161" s="35" t="s">
-        <v>5432</v>
+        <v>5433</v>
       </c>
       <c r="E161" s="35" t="s">
         <v>4068</v>
@@ -74710,7 +74713,7 @@
         <v>3962</v>
       </c>
       <c r="D162" s="35" t="s">
-        <v>5432</v>
+        <v>5433</v>
       </c>
       <c r="E162" s="35" t="s">
         <v>4037</v>
@@ -74726,7 +74729,7 @@
         <v>3962</v>
       </c>
       <c r="D163" s="35" t="s">
-        <v>5432</v>
+        <v>5433</v>
       </c>
       <c r="E163" s="35" t="s">
         <v>4047</v>
@@ -74742,7 +74745,7 @@
         <v>3962</v>
       </c>
       <c r="D164" s="35" t="s">
-        <v>5432</v>
+        <v>5433</v>
       </c>
       <c r="E164" s="35" t="s">
         <v>3994</v>
@@ -74760,7 +74763,7 @@
         <v>3970</v>
       </c>
       <c r="D165" s="35" t="s">
-        <v>5432</v>
+        <v>5433</v>
       </c>
       <c r="E165" s="35" t="s">
         <v>331</v>
@@ -74776,7 +74779,7 @@
         <v>1307</v>
       </c>
       <c r="D166" s="35" t="s">
-        <v>5433</v>
+        <v>5434</v>
       </c>
       <c r="E166" s="35" t="s">
         <v>1205</v>
@@ -74792,7 +74795,7 @@
         <v>1307</v>
       </c>
       <c r="D167" s="35" t="s">
-        <v>5433</v>
+        <v>5434</v>
       </c>
       <c r="E167" s="35" t="s">
         <v>1325</v>
@@ -74888,7 +74891,7 @@
         <v>2367</v>
       </c>
       <c r="D173" s="35" t="s">
-        <v>5434</v>
+        <v>5435</v>
       </c>
       <c r="E173" s="35" t="s">
         <v>2366</v>
@@ -74904,7 +74907,7 @@
         <v>833</v>
       </c>
       <c r="D174" s="35" t="s">
-        <v>5435</v>
+        <v>5436</v>
       </c>
       <c r="E174" s="35" t="s">
         <v>815</v>
@@ -74920,7 +74923,7 @@
         <v>847</v>
       </c>
       <c r="D175" s="35" t="s">
-        <v>5435</v>
+        <v>5436</v>
       </c>
       <c r="E175" s="35" t="s">
         <v>815</v>
@@ -74936,7 +74939,7 @@
         <v>3645</v>
       </c>
       <c r="D176" s="35" t="s">
-        <v>5435</v>
+        <v>5436</v>
       </c>
       <c r="E176" s="35" t="s">
         <v>3633</v>
@@ -74952,7 +74955,7 @@
         <v>1669</v>
       </c>
       <c r="D177" s="35" t="s">
-        <v>5435</v>
+        <v>5436</v>
       </c>
       <c r="E177" s="35" t="s">
         <v>919</v>
@@ -74970,7 +74973,7 @@
         <v>3669</v>
       </c>
       <c r="D178" s="35" t="s">
-        <v>5436</v>
+        <v>5437</v>
       </c>
       <c r="E178" s="35" t="s">
         <v>3538</v>
@@ -74986,7 +74989,7 @@
         <v>944</v>
       </c>
       <c r="D179" s="35" t="s">
-        <v>5436</v>
+        <v>5437</v>
       </c>
       <c r="E179" s="35" t="s">
         <v>815</v>
@@ -75006,7 +75009,7 @@
         <v>944</v>
       </c>
       <c r="D180" s="35" t="s">
-        <v>5436</v>
+        <v>5437</v>
       </c>
       <c r="E180" s="35" t="s">
         <v>625</v>
@@ -75022,7 +75025,7 @@
         <v>902</v>
       </c>
       <c r="D181" s="35" t="s">
-        <v>5437</v>
+        <v>5438</v>
       </c>
       <c r="E181" s="35" t="s">
         <v>892</v>
@@ -75038,7 +75041,7 @@
         <v>1105</v>
       </c>
       <c r="D182" s="35" t="s">
-        <v>5438</v>
+        <v>5439</v>
       </c>
       <c r="E182" s="35" t="s">
         <v>1080</v>
@@ -75054,7 +75057,7 @@
         <v>1105</v>
       </c>
       <c r="D183" s="35" t="s">
-        <v>5438</v>
+        <v>5439</v>
       </c>
       <c r="E183" s="35" t="s">
         <v>3715</v>
@@ -75067,10 +75070,10 @@
       <c r="A184" s="33"/>
       <c r="B184" s="33"/>
       <c r="C184" s="34" t="s">
-        <v>5439</v>
+        <v>5440</v>
       </c>
       <c r="D184" s="35" t="s">
-        <v>5440</v>
+        <v>5441</v>
       </c>
       <c r="E184" s="35" t="s">
         <v>1080</v>
@@ -75083,10 +75086,10 @@
       <c r="A185" s="33"/>
       <c r="B185" s="33"/>
       <c r="C185" s="34" t="s">
-        <v>5439</v>
+        <v>5440</v>
       </c>
       <c r="D185" s="35" t="s">
-        <v>5440</v>
+        <v>5441</v>
       </c>
       <c r="E185" s="35" t="s">
         <v>3715</v>
@@ -75103,10 +75106,10 @@
         <v>563</v>
       </c>
       <c r="C186" s="34" t="s">
+        <v>5442</v>
+      </c>
+      <c r="D186" s="35" t="s">
         <v>5441</v>
-      </c>
-      <c r="D186" s="35" t="s">
-        <v>5440</v>
       </c>
       <c r="E186" s="35" t="s">
         <v>1080</v>
@@ -75122,7 +75125,7 @@
         <v>3726</v>
       </c>
       <c r="D187" s="35" t="s">
-        <v>5440</v>
+        <v>5441</v>
       </c>
       <c r="E187" s="35" t="s">
         <v>3715</v>
@@ -75139,10 +75142,10 @@
         <v>563</v>
       </c>
       <c r="C188" s="34" t="s">
-        <v>5442</v>
+        <v>5443</v>
       </c>
       <c r="D188" s="35" t="s">
-        <v>5440</v>
+        <v>5441</v>
       </c>
       <c r="E188" s="35" t="s">
         <v>1080</v>
@@ -75159,10 +75162,10 @@
         <v>563</v>
       </c>
       <c r="C189" s="34" t="s">
-        <v>5443</v>
+        <v>5444</v>
       </c>
       <c r="D189" s="35" t="s">
-        <v>5440</v>
+        <v>5441</v>
       </c>
       <c r="E189" s="35" t="s">
         <v>1080</v>
@@ -75178,7 +75181,7 @@
         <v>1099</v>
       </c>
       <c r="D190" s="35" t="s">
-        <v>5440</v>
+        <v>5441</v>
       </c>
       <c r="E190" s="35" t="s">
         <v>1080</v>
@@ -75194,7 +75197,7 @@
         <v>1073</v>
       </c>
       <c r="D191" s="35" t="s">
-        <v>5444</v>
+        <v>5445</v>
       </c>
       <c r="E191" s="35" t="s">
         <v>1048</v>
@@ -75210,7 +75213,7 @@
         <v>1073</v>
       </c>
       <c r="D192" s="35" t="s">
-        <v>5444</v>
+        <v>5445</v>
       </c>
       <c r="E192" s="35" t="s">
         <v>3698</v>
@@ -75223,10 +75226,10 @@
       <c r="A193" s="33"/>
       <c r="B193" s="33"/>
       <c r="C193" s="34" t="s">
-        <v>5445</v>
+        <v>5446</v>
       </c>
       <c r="D193" s="35" t="s">
-        <v>5446</v>
+        <v>5447</v>
       </c>
       <c r="E193" s="35" t="s">
         <v>1048</v>
@@ -75239,10 +75242,10 @@
       <c r="A194" s="33"/>
       <c r="B194" s="33"/>
       <c r="C194" s="34" t="s">
-        <v>5445</v>
+        <v>5446</v>
       </c>
       <c r="D194" s="35" t="s">
-        <v>5446</v>
+        <v>5447</v>
       </c>
       <c r="E194" s="35" t="s">
         <v>3698</v>
@@ -75259,10 +75262,10 @@
         <v>563</v>
       </c>
       <c r="C195" s="34" t="s">
+        <v>5448</v>
+      </c>
+      <c r="D195" s="35" t="s">
         <v>5447</v>
-      </c>
-      <c r="D195" s="35" t="s">
-        <v>5446</v>
       </c>
       <c r="E195" s="35" t="s">
         <v>1048</v>
@@ -75278,7 +75281,7 @@
         <v>3709</v>
       </c>
       <c r="D196" s="35" t="s">
-        <v>5446</v>
+        <v>5447</v>
       </c>
       <c r="E196" s="35" t="s">
         <v>3698</v>
@@ -75295,10 +75298,10 @@
         <v>563</v>
       </c>
       <c r="C197" s="34" t="s">
-        <v>5448</v>
+        <v>5449</v>
       </c>
       <c r="D197" s="35" t="s">
-        <v>5446</v>
+        <v>5447</v>
       </c>
       <c r="E197" s="35" t="s">
         <v>1048</v>
@@ -75315,10 +75318,10 @@
         <v>563</v>
       </c>
       <c r="C198" s="34" t="s">
-        <v>5449</v>
+        <v>5450</v>
       </c>
       <c r="D198" s="35" t="s">
-        <v>5446</v>
+        <v>5447</v>
       </c>
       <c r="E198" s="35" t="s">
         <v>1048</v>
@@ -75334,7 +75337,7 @@
         <v>1067</v>
       </c>
       <c r="D199" s="35" t="s">
-        <v>5446</v>
+        <v>5447</v>
       </c>
       <c r="E199" s="35" t="s">
         <v>1048</v>
@@ -75400,7 +75403,7 @@
         <v>3664</v>
       </c>
       <c r="D203" s="35" t="s">
-        <v>5450</v>
+        <v>5451</v>
       </c>
       <c r="E203" s="35" t="s">
         <v>3538</v>
@@ -75420,7 +75423,7 @@
         <v>937</v>
       </c>
       <c r="D204" s="35" t="s">
-        <v>5450</v>
+        <v>5451</v>
       </c>
       <c r="E204" s="35" t="s">
         <v>625</v>
@@ -75436,7 +75439,7 @@
         <v>937</v>
       </c>
       <c r="D205" s="35" t="s">
-        <v>5450</v>
+        <v>5451</v>
       </c>
       <c r="E205" s="35" t="s">
         <v>975</v>
@@ -75452,7 +75455,7 @@
         <v>937</v>
       </c>
       <c r="D206" s="35" t="s">
-        <v>5450</v>
+        <v>5451</v>
       </c>
       <c r="E206" s="35" t="s">
         <v>998</v>
@@ -75520,7 +75523,7 @@
         <v>711</v>
       </c>
       <c r="D210" s="35" t="s">
-        <v>5451</v>
+        <v>5452</v>
       </c>
       <c r="E210" s="35" t="s">
         <v>647</v>
@@ -75540,7 +75543,7 @@
         <v>711</v>
       </c>
       <c r="D211" s="35" t="s">
-        <v>5451</v>
+        <v>5452</v>
       </c>
       <c r="E211" s="35" t="s">
         <v>647</v>
@@ -75560,7 +75563,7 @@
         <v>711</v>
       </c>
       <c r="D212" s="35" t="s">
-        <v>5451</v>
+        <v>5452</v>
       </c>
       <c r="E212" s="35" t="s">
         <v>715</v>
@@ -75576,7 +75579,7 @@
         <v>650</v>
       </c>
       <c r="D213" s="35" t="s">
-        <v>5452</v>
+        <v>5453</v>
       </c>
       <c r="E213" s="35" t="s">
         <v>647</v>
@@ -75592,7 +75595,7 @@
         <v>1998</v>
       </c>
       <c r="D214" s="35" t="s">
-        <v>5452</v>
+        <v>5453</v>
       </c>
       <c r="E214" s="35" t="s">
         <v>1995</v>
@@ -75608,7 +75611,7 @@
         <v>345</v>
       </c>
       <c r="D215" s="35" t="s">
-        <v>5452</v>
+        <v>5453</v>
       </c>
       <c r="E215" s="35" t="s">
         <v>331</v>
@@ -75624,7 +75627,7 @@
         <v>3553</v>
       </c>
       <c r="D216" s="35" t="s">
-        <v>5452</v>
+        <v>5453</v>
       </c>
       <c r="E216" s="35" t="s">
         <v>3550</v>
@@ -75640,7 +75643,7 @@
         <v>341</v>
       </c>
       <c r="D217" s="35" t="s">
-        <v>5452</v>
+        <v>5453</v>
       </c>
       <c r="E217" s="35" t="s">
         <v>331</v>
@@ -75660,7 +75663,7 @@
         <v>2149</v>
       </c>
       <c r="D218" s="35" t="s">
-        <v>5452</v>
+        <v>5453</v>
       </c>
       <c r="E218" s="35" t="s">
         <v>2119</v>
@@ -75676,7 +75679,7 @@
         <v>151</v>
       </c>
       <c r="D219" s="35" t="s">
-        <v>5452</v>
+        <v>5453</v>
       </c>
       <c r="E219" s="35" t="s">
         <v>41</v>
@@ -75692,7 +75695,7 @@
         <v>144</v>
       </c>
       <c r="D220" s="35" t="s">
-        <v>5452</v>
+        <v>5453</v>
       </c>
       <c r="E220" s="35" t="s">
         <v>41</v>
@@ -75708,7 +75711,7 @@
         <v>2638</v>
       </c>
       <c r="D221" s="35" t="s">
-        <v>5452</v>
+        <v>5453</v>
       </c>
       <c r="E221" s="35" t="s">
         <v>2612</v>
@@ -75724,7 +75727,7 @@
         <v>965</v>
       </c>
       <c r="D222" s="35" t="s">
-        <v>5452</v>
+        <v>5453</v>
       </c>
       <c r="E222" s="35" t="s">
         <v>951</v>
@@ -75740,7 +75743,7 @@
         <v>621</v>
       </c>
       <c r="D223" s="35" t="s">
-        <v>5452</v>
+        <v>5453</v>
       </c>
       <c r="E223" s="35" t="s">
         <v>594</v>
@@ -75756,7 +75759,7 @@
         <v>1973</v>
       </c>
       <c r="D224" s="35" t="s">
-        <v>5452</v>
+        <v>5453</v>
       </c>
       <c r="E224" s="35" t="s">
         <v>1953</v>
@@ -75772,7 +75775,7 @@
         <v>105</v>
       </c>
       <c r="D225" s="35" t="s">
-        <v>5452</v>
+        <v>5453</v>
       </c>
       <c r="E225" s="35" t="s">
         <v>41</v>
@@ -75788,7 +75791,7 @@
         <v>105</v>
       </c>
       <c r="D226" s="35" t="s">
-        <v>5452</v>
+        <v>5453</v>
       </c>
       <c r="E226" s="35" t="s">
         <v>2612</v>
@@ -75804,7 +75807,7 @@
         <v>3912</v>
       </c>
       <c r="D227" s="35" t="s">
-        <v>5452</v>
+        <v>5453</v>
       </c>
       <c r="E227" s="35" t="s">
         <v>3904</v>
@@ -75824,7 +75827,7 @@
         <v>286</v>
       </c>
       <c r="D228" s="35" t="s">
-        <v>5452</v>
+        <v>5453</v>
       </c>
       <c r="E228" s="35" t="s">
         <v>280</v>
@@ -75840,7 +75843,7 @@
         <v>3543</v>
       </c>
       <c r="D229" s="35" t="s">
-        <v>5452</v>
+        <v>5453</v>
       </c>
       <c r="E229" s="35" t="s">
         <v>3540</v>
@@ -75856,13 +75859,13 @@
         <v>2082</v>
       </c>
       <c r="D230" s="35" t="s">
-        <v>5452</v>
+        <v>5453</v>
       </c>
       <c r="E230" s="35" t="s">
-        <v>5418</v>
+        <v>5419</v>
       </c>
       <c r="F230" s="34" t="s">
-        <v>5419</v>
+        <v>5420</v>
       </c>
     </row>
     <row r="231">
@@ -75872,7 +75875,7 @@
         <v>2124</v>
       </c>
       <c r="D231" s="35" t="s">
-        <v>5452</v>
+        <v>5453</v>
       </c>
       <c r="E231" s="35" t="s">
         <v>2119</v>
@@ -75888,7 +75891,7 @@
         <v>2290</v>
       </c>
       <c r="D232" s="35" t="s">
-        <v>5452</v>
+        <v>5453</v>
       </c>
       <c r="E232" s="35" t="s">
         <v>2282</v>
@@ -75904,7 +75907,7 @@
         <v>3353</v>
       </c>
       <c r="D233" s="35" t="s">
-        <v>5452</v>
+        <v>5453</v>
       </c>
       <c r="E233" s="35" t="s">
         <v>3348</v>
@@ -75920,7 +75923,7 @@
         <v>3534</v>
       </c>
       <c r="D234" s="35" t="s">
-        <v>5452</v>
+        <v>5453</v>
       </c>
       <c r="E234" s="35" t="s">
         <v>3525</v>
@@ -75936,7 +75939,7 @@
         <v>642</v>
       </c>
       <c r="D235" s="35" t="s">
-        <v>5452</v>
+        <v>5453</v>
       </c>
       <c r="E235" s="35" t="s">
         <v>627</v>
@@ -75952,7 +75955,7 @@
         <v>3547</v>
       </c>
       <c r="D236" s="35" t="s">
-        <v>5452</v>
+        <v>5453</v>
       </c>
       <c r="E236" s="35" t="s">
         <v>3540</v>
@@ -75968,7 +75971,7 @@
         <v>635</v>
       </c>
       <c r="D237" s="35" t="s">
-        <v>5452</v>
+        <v>5453</v>
       </c>
       <c r="E237" s="35" t="s">
         <v>627</v>
@@ -75984,7 +75987,7 @@
         <v>2387</v>
       </c>
       <c r="D238" s="35" t="s">
-        <v>5452</v>
+        <v>5453</v>
       </c>
       <c r="E238" s="35" t="s">
         <v>2366</v>
@@ -76000,7 +76003,7 @@
         <v>89</v>
       </c>
       <c r="D239" s="35" t="s">
-        <v>5452</v>
+        <v>5453</v>
       </c>
       <c r="E239" s="35" t="s">
         <v>41</v>
@@ -76016,7 +76019,7 @@
         <v>2740</v>
       </c>
       <c r="D240" s="35" t="s">
-        <v>5452</v>
+        <v>5453</v>
       </c>
       <c r="E240" s="35" t="s">
         <v>2726</v>
@@ -76036,7 +76039,7 @@
         <v>2092</v>
       </c>
       <c r="D241" s="35" t="s">
-        <v>5452</v>
+        <v>5453</v>
       </c>
       <c r="E241" s="35" t="s">
         <v>2086</v>
@@ -76054,7 +76057,7 @@
         <v>3951</v>
       </c>
       <c r="D242" s="35" t="s">
-        <v>5452</v>
+        <v>5453</v>
       </c>
       <c r="E242" s="35" t="s">
         <v>3936</v>
@@ -76074,7 +76077,7 @@
         <v>731</v>
       </c>
       <c r="D243" s="35" t="s">
-        <v>5453</v>
+        <v>5454</v>
       </c>
       <c r="E243" s="35" t="s">
         <v>647</v>
@@ -76090,7 +76093,7 @@
         <v>820</v>
       </c>
       <c r="D244" s="35" t="s">
-        <v>5454</v>
+        <v>5455</v>
       </c>
       <c r="E244" s="35" t="s">
         <v>815</v>
@@ -76106,7 +76109,7 @@
         <v>3636</v>
       </c>
       <c r="D245" s="35" t="s">
-        <v>5454</v>
+        <v>5455</v>
       </c>
       <c r="E245" s="35" t="s">
         <v>3633</v>
@@ -76122,7 +76125,7 @@
         <v>827</v>
       </c>
       <c r="D246" s="35" t="s">
-        <v>5454</v>
+        <v>5455</v>
       </c>
       <c r="E246" s="35" t="s">
         <v>815</v>
@@ -76138,7 +76141,7 @@
         <v>3641</v>
       </c>
       <c r="D247" s="35" t="s">
-        <v>5454</v>
+        <v>5455</v>
       </c>
       <c r="E247" s="35" t="s">
         <v>3633</v>
@@ -76151,10 +76154,10 @@
       <c r="A248" s="33"/>
       <c r="B248" s="33"/>
       <c r="C248" s="34" t="s">
-        <v>5455</v>
+        <v>5456</v>
       </c>
       <c r="D248" s="35" t="s">
-        <v>5456</v>
+        <v>5457</v>
       </c>
       <c r="E248" s="35" t="s">
         <v>815</v>
@@ -76167,10 +76170,10 @@
       <c r="A249" s="33"/>
       <c r="B249" s="33"/>
       <c r="C249" s="34" t="s">
+        <v>5458</v>
+      </c>
+      <c r="D249" s="35" t="s">
         <v>5457</v>
-      </c>
-      <c r="D249" s="35" t="s">
-        <v>5456</v>
       </c>
       <c r="E249" s="35" t="s">
         <v>3633</v>
@@ -76187,10 +76190,10 @@
         <v>282</v>
       </c>
       <c r="C250" s="34" t="s">
-        <v>5458</v>
+        <v>5459</v>
       </c>
       <c r="D250" s="35" t="s">
-        <v>5459</v>
+        <v>5460</v>
       </c>
       <c r="E250" s="35" t="s">
         <v>1205</v>
@@ -76203,10 +76206,10 @@
       <c r="A251" s="33"/>
       <c r="B251" s="33"/>
       <c r="C251" s="34" t="s">
-        <v>5460</v>
+        <v>5461</v>
       </c>
       <c r="D251" s="35" t="s">
-        <v>5461</v>
+        <v>5462</v>
       </c>
       <c r="E251" s="35" t="s">
         <v>2117</v>
@@ -76222,7 +76225,7 @@
         <v>2247</v>
       </c>
       <c r="D252" s="35" t="s">
-        <v>5461</v>
+        <v>5462</v>
       </c>
       <c r="E252" s="35" t="s">
         <v>2117</v>
@@ -76238,7 +76241,7 @@
         <v>2251</v>
       </c>
       <c r="D253" s="35" t="s">
-        <v>5461</v>
+        <v>5462</v>
       </c>
       <c r="E253" s="35" t="s">
         <v>2117</v>
@@ -76254,7 +76257,7 @@
         <v>455</v>
       </c>
       <c r="D254" s="35" t="s">
-        <v>5462</v>
+        <v>5463</v>
       </c>
       <c r="E254" s="35" t="s">
         <v>418</v>
@@ -76270,7 +76273,7 @@
         <v>419</v>
       </c>
       <c r="D255" s="35" t="s">
-        <v>5462</v>
+        <v>5463</v>
       </c>
       <c r="E255" s="35" t="s">
         <v>418</v>
@@ -76286,7 +76289,7 @@
         <v>771</v>
       </c>
       <c r="D256" s="35" t="s">
-        <v>5462</v>
+        <v>5463</v>
       </c>
       <c r="E256" s="35" t="s">
         <v>770</v>
@@ -76306,7 +76309,7 @@
         <v>771</v>
       </c>
       <c r="D257" s="35" t="s">
-        <v>5462</v>
+        <v>5463</v>
       </c>
       <c r="E257" s="35" t="s">
         <v>770</v>
@@ -76322,7 +76325,7 @@
         <v>3618</v>
       </c>
       <c r="D258" s="35" t="s">
-        <v>5462</v>
+        <v>5463</v>
       </c>
       <c r="E258" s="35" t="s">
         <v>3603</v>
@@ -77604,7 +77607,7 @@
         <v>595</v>
       </c>
       <c r="D331" s="35" t="s">
-        <v>5463</v>
+        <v>5464</v>
       </c>
       <c r="E331" s="35" t="s">
         <v>919</v>
@@ -77624,7 +77627,7 @@
         <v>595</v>
       </c>
       <c r="D332" s="35" t="s">
-        <v>5464</v>
+        <v>5465</v>
       </c>
       <c r="E332" s="35" t="s">
         <v>1236</v>
@@ -77917,12 +77920,12 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="36" t="s">
-        <v>5465</v>
+        <v>5466</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="37" t="s">
-        <v>5466</v>
+        <v>5467</v>
       </c>
     </row>
   </sheetData>
@@ -77944,154 +77947,154 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="38" t="s">
-        <v>5467</v>
+        <v>5468</v>
       </c>
       <c r="E1" s="39" t="s">
-        <v>5468</v>
+        <v>5469</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="40"/>
       <c r="E2" s="41" t="s">
-        <v>5469</v>
+        <v>5470</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="42" t="s">
-        <v>5470</v>
+        <v>5471</v>
       </c>
       <c r="E3" s="43" t="s">
-        <v>5471</v>
+        <v>5472</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="24" t="s">
-        <v>5472</v>
+        <v>5473</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>5473</v>
+        <v>5474</v>
       </c>
       <c r="E4" s="43" t="s">
-        <v>5474</v>
+        <v>5475</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="38" t="s">
-        <v>5475</v>
+        <v>5476</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>5476</v>
+        <v>5477</v>
       </c>
       <c r="E5" s="44" t="s">
-        <v>5477</v>
+        <v>5478</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="45" t="s">
-        <v>5478</v>
+        <v>5479</v>
       </c>
       <c r="B6" s="10" t="s">
-        <v>5479</v>
+        <v>5480</v>
       </c>
       <c r="E6" s="43" t="s">
-        <v>5480</v>
+        <v>5481</v>
       </c>
     </row>
     <row r="7">
       <c r="E7" s="46" t="s">
-        <v>5481</v>
+        <v>5482</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="42" t="s">
-        <v>5482</v>
+        <v>5483</v>
       </c>
       <c r="E8" s="46" t="s">
-        <v>5483</v>
+        <v>5484</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="47" t="s">
-        <v>5484</v>
+        <v>5485</v>
       </c>
       <c r="B9" s="40" t="s">
-        <v>5485</v>
+        <v>5486</v>
       </c>
       <c r="E9" s="44" t="s">
-        <v>5486</v>
+        <v>5487</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="40" t="s">
-        <v>5487</v>
+        <v>5488</v>
       </c>
       <c r="B10" s="40" t="s">
         <v>0</v>
       </c>
       <c r="E10" s="48" t="s">
-        <v>5488</v>
+        <v>5489</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="49" t="s">
-        <v>5489</v>
+        <v>5490</v>
       </c>
       <c r="B11" s="40" t="s">
-        <v>5490</v>
+        <v>5491</v>
       </c>
       <c r="E11" s="50" t="s">
-        <v>5491</v>
+        <v>5492</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="51" t="s">
-        <v>5489</v>
+        <v>5490</v>
       </c>
       <c r="B12" s="40" t="s">
-        <v>5492</v>
+        <v>5493</v>
       </c>
       <c r="E12" s="52" t="s">
-        <v>5493</v>
+        <v>5494</v>
       </c>
     </row>
     <row r="13">
       <c r="E13" s="53" t="s">
-        <v>5494</v>
+        <v>5495</v>
       </c>
     </row>
     <row r="14">
       <c r="E14" s="54" t="s">
-        <v>5495</v>
+        <v>5496</v>
       </c>
     </row>
     <row r="15">
       <c r="E15" s="55" t="s">
-        <v>5496</v>
+        <v>5497</v>
       </c>
     </row>
     <row r="16">
       <c r="E16" s="56" t="s">
-        <v>5497</v>
+        <v>5498</v>
       </c>
     </row>
     <row r="17">
       <c r="E17" s="56" t="s">
-        <v>5498</v>
+        <v>5499</v>
       </c>
     </row>
     <row r="18">
       <c r="E18" s="52" t="s">
-        <v>5499</v>
+        <v>5500</v>
       </c>
     </row>
     <row r="19">
       <c r="E19" s="43" t="s">
-        <v>5500</v>
+        <v>5501</v>
       </c>
     </row>
     <row r="20">
       <c r="E20" s="57" t="s">
-        <v>5501</v>
+        <v>5502</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix: update ePO 5 package CMs for fixes on further XPath conditions
</commit_message>
<xml_diff>
--- a/mappings/package_eforms_sdk1.3_epo5.2/transformation/conceptual_mappings.xlsx
+++ b/mappings/package_eforms_sdk1.3_epo5.2/transformation/conceptual_mappings.xlsx
@@ -2584,7 +2584,7 @@
     <t>MG-Duration-hasEstimatedDuration-DynamicPurchaseSystemTechnique-usesTechnique-Lot</t>
   </si>
   <si>
-    <t>/*/cac:ProcurementProjectLot[cbc:ID/@schemeName='Lot']/cac:TenderingProcess/cac:ContractingSystem[cbc:ContractingSystemTypeCode/@listName='dps-usage' and not(text()='none')]</t>
+    <t>/*/cac:ProcurementProjectLot[cbc:ID/@schemeName='Lot']/cac:TenderingProcess/cac:ContractingSystem[cbc:ContractingSystemTypeCode/@listName='dps-usage' and not(cbc:ContractingSystemTypeCode/text()='none'))]</t>
   </si>
   <si>
     <t>epo:Lot / epo:DynamicPurchaseSystemTechnique / time:Duration / xsd:decimal</t>
@@ -2596,7 +2596,7 @@
     <t xml:space="preserve">We need an alternative mapping here in case we have a DPS. We also need an xpath on top, </t>
   </si>
   <si>
-    <t>/*/cac:ProcurementProjectLot[cbc:ID/@schemeName='Lot']/cac:TenderingProcess/cac:ContractingSystem[cbc:ContractingSystemTypeCode/@listName='dps-usage' and not(text()='none')] and cbc:DurationMeasure[@unitCode='DAY']</t>
+    <t>/*/cac:ProcurementProjectLot[cbc:ID/@schemeName='Lot']/cac:TenderingProcess/cac:ContractingSystem[cbc:ContractingSystemTypeCode/@listName='dps-usage' and not(cbc:ContractingSystemTypeCode/text()='none'))] and cbc:DurationMeasure[@unitCode='DAY']</t>
   </si>
   <si>
     <t>epo:Lot / epo:DynamicPurchaseSystemTechnique / time:Duration / time:TemporalUnit</t>
@@ -2605,19 +2605,19 @@
     <t>?this epo:usesTechnique / epo:hasEstimatedDuration / time:unitType time:unitDay .</t>
   </si>
   <si>
-    <t>/*/cac:ProcurementProjectLot[cbc:ID/@schemeName='Lot']/cac:TenderingProcess/cac:ContractingSystem[cbc:ContractingSystemTypeCode/@listName='dps-usage' and not(text()='none')] and cbc:DurationMeasure[@unitCode='WEEK']</t>
+    <t>/*/cac:ProcurementProjectLot[cbc:ID/@schemeName='Lot']/cac:TenderingProcess/cac:ContractingSystem[cbc:ContractingSystemTypeCode/@listName='dps-usage' and not(cbc:ContractingSystemTypeCode/text()='none'))] and cbc:DurationMeasure[@unitCode='WEEK']</t>
   </si>
   <si>
     <t>?this epo:usesTechnique / epo:hasEstimatedDuration / time:unitType time:unitWeek .</t>
   </si>
   <si>
-    <t>/*/cac:ProcurementProjectLot[cbc:ID/@schemeName='Lot']/cac:TenderingProcess/cac:ContractingSystem[cbc:ContractingSystemTypeCode/@listName='dps-usage' and not(text()='none')] and cbc:DurationMeasure[@unitCode='MONTH']</t>
+    <t>/*/cac:ProcurementProjectLot[cbc:ID/@schemeName='Lot']/cac:TenderingProcess/cac:ContractingSystem[cbc:ContractingSystemTypeCode/@listName='dps-usage' and not(cbc:ContractingSystemTypeCode/text()='none'))] and cbc:DurationMeasure[@unitCode='MONTH']</t>
   </si>
   <si>
     <t>?this epo:usesTechnique / epo:hasEstimatedDuration / time:unitType time:unitMonth .</t>
   </si>
   <si>
-    <t>/*/cac:ProcurementProjectLot[cbc:ID/@schemeName='Lot']/cac:TenderingProcess/cac:ContractingSystem[cbc:ContractingSystemTypeCode/@listName='dps-usage' and not(text()='none')] and cbc:DurationMeasure[@unitCode='YEAR']</t>
+    <t>/*/cac:ProcurementProjectLot[cbc:ID/@schemeName='Lot']/cac:TenderingProcess/cac:ContractingSystem[cbc:ContractingSystemTypeCode/@listName='dps-usage' and not(cbc:ContractingSystemTypeCode/text()='none'))] and cbc:DurationMeasure[@unitCode='YEAR']</t>
   </si>
   <si>
     <t>?this epo:usesTechnique / epo:hasEstimatedDuration / time:unitType time:unitYear .</t>

</xml_diff>

<commit_message>
fix: update package CMs for erroneous class path
</commit_message>
<xml_diff>
--- a/mappings/package_eforms_sdk1.3_epo5.2/transformation/conceptual_mappings.xlsx
+++ b/mappings/package_eforms_sdk1.3_epo5.2/transformation/conceptual_mappings.xlsx
@@ -2584,7 +2584,7 @@
     <t>MG-Duration-hasEstimatedDuration-DynamicPurchaseSystemTechnique-usesTechnique-Lot</t>
   </si>
   <si>
-    <t>/*/cac:ProcurementProjectLot[cbc:ID/@schemeName='Lot']/cac:TenderingProcess/cac:ContractingSystem[cbc:ContractingSystemTypeCode/@listName='dps-usage' and not(cbc:ContractingSystemTypeCode/text()='none'))]</t>
+    <t>exists(../../cac:TenderingProcess/cac:ContractingSystem[cbc:ContractingSystemTypeCode/@listName='dps-usage']/cbc:ContractingSystemTypeCode[not(text()='none')])</t>
   </si>
   <si>
     <t>epo:Lot / epo:DynamicPurchaseSystemTechnique / time:Duration / xsd:decimal</t>
@@ -2596,7 +2596,7 @@
     <t xml:space="preserve">We need an alternative mapping here in case we have a DPS. We also need an xpath on top, </t>
   </si>
   <si>
-    <t>/*/cac:ProcurementProjectLot[cbc:ID/@schemeName='Lot']/cac:TenderingProcess/cac:ContractingSystem[cbc:ContractingSystemTypeCode/@listName='dps-usage' and not(cbc:ContractingSystemTypeCode/text()='none'))] and cbc:DurationMeasure[@unitCode='DAY']</t>
+    <t>exists(../../cac:TenderingProcess/cac:ContractingSystem[cbc:ContractingSystemTypeCode/@listName='dps-usage']/cbc:ContractingSystemTypeCode[not(text()='none')]) and cbc:DurationMeasure/@unitCode='DAY'</t>
   </si>
   <si>
     <t>epo:Lot / epo:DynamicPurchaseSystemTechnique / time:Duration / time:TemporalUnit</t>
@@ -2605,19 +2605,19 @@
     <t>?this epo:usesTechnique / epo:hasEstimatedDuration / time:unitType time:unitDay .</t>
   </si>
   <si>
-    <t>/*/cac:ProcurementProjectLot[cbc:ID/@schemeName='Lot']/cac:TenderingProcess/cac:ContractingSystem[cbc:ContractingSystemTypeCode/@listName='dps-usage' and not(cbc:ContractingSystemTypeCode/text()='none'))] and cbc:DurationMeasure[@unitCode='WEEK']</t>
+    <t>exists(../../cac:TenderingProcess/cac:ContractingSystem[cbc:ContractingSystemTypeCode/@listName='dps-usage']/cbc:ContractingSystemTypeCode[not(text()='none')]) and cbc:DurationMeasure/@unitCode='WEEK'</t>
   </si>
   <si>
     <t>?this epo:usesTechnique / epo:hasEstimatedDuration / time:unitType time:unitWeek .</t>
   </si>
   <si>
-    <t>/*/cac:ProcurementProjectLot[cbc:ID/@schemeName='Lot']/cac:TenderingProcess/cac:ContractingSystem[cbc:ContractingSystemTypeCode/@listName='dps-usage' and not(cbc:ContractingSystemTypeCode/text()='none'))] and cbc:DurationMeasure[@unitCode='MONTH']</t>
+    <t>exists(../../cac:TenderingProcess/cac:ContractingSystem[cbc:ContractingSystemTypeCode/@listName='dps-usage']/cbc:ContractingSystemTypeCode[not(text()='none')]) and cbc:DurationMeasure/@unitCode='MONTH'</t>
   </si>
   <si>
     <t>?this epo:usesTechnique / epo:hasEstimatedDuration / time:unitType time:unitMonth .</t>
   </si>
   <si>
-    <t>/*/cac:ProcurementProjectLot[cbc:ID/@schemeName='Lot']/cac:TenderingProcess/cac:ContractingSystem[cbc:ContractingSystemTypeCode/@listName='dps-usage' and not(cbc:ContractingSystemTypeCode/text()='none'))] and cbc:DurationMeasure[@unitCode='YEAR']</t>
+    <t>exists(../../cac:TenderingProcess/cac:ContractingSystem[cbc:ContractingSystemTypeCode/@listName='dps-usage']/cbc:ContractingSystemTypeCode[not(text()='none')]) and cbc:DurationMeasure/@unitCode='YEAR'</t>
   </si>
   <si>
     <t>?this epo:usesTechnique / epo:hasEstimatedDuration / time:unitType time:unitYear .</t>
@@ -15463,8 +15463,7 @@
     <t>epo:ContractLotCompletionInformation / epo:MonetaryValue / at-voc:currency</t>
   </si>
   <si>
-    <t xml:space="preserve">
-?this  epo:providesContractTotalPaymentValue / epo:hasCurrency ?value .</t>
+    <t>?this  epo:providesContractTotalPaymentValue / epo:hasCurrency ?value .</t>
   </si>
   <si>
     <t>BT-780-Tender-Language</t>

</xml_diff>

<commit_message>
feat: update package CMs for prefix corrections cbc -> efbc
</commit_message>
<xml_diff>
--- a/mappings/package_eforms_sdk1.3_epo5.2/transformation/conceptual_mappings.xlsx
+++ b/mappings/package_eforms_sdk1.3_epo5.2/transformation/conceptual_mappings.xlsx
@@ -12317,31 +12317,31 @@
     <t>/*/ext:UBLExtensions/ext:UBLExtension/ext:ExtensionContent/efext:EformsExtension/efac:NoticeResult/efac:LotTender/efac:ContractTerm[not(efbc:TermCode/text()='all-rev-tic')][efbc:TermCode/@listName='contract-detail']/efbc:TermDescription</t>
   </si>
   <si>
-    <t>cbc:TermCode[@listName='contract-detail']/text()='cost-comp'</t>
+    <t>efbc:TermCode[@listName='contract-detail']/text()='cost-comp'</t>
   </si>
   <si>
     <t>?this epo:hasCompensationCostParametersDescription ?value .</t>
   </si>
   <si>
-    <t>cbc:TermCode[@listName='contract-detail']/text()='other'</t>
+    <t>efbc:TermCode[@listName='contract-detail']/text()='other'</t>
   </si>
   <si>
     <t>?this epo:hasParticularConditionsDescription ?value .</t>
   </si>
   <si>
-    <t>cbc:TermCode[@listName='contract-detail']/text()='exc-right'</t>
+    <t>efbc:TermCode[@listName='contract-detail']/text()='exc-right'</t>
   </si>
   <si>
     <t>?this epo:hasGrantedExclusiveRightsDescription ?value .</t>
   </si>
   <si>
-    <t>cbc:TermCode[@listName='contract-detail']/text()='publ-ser-obl'</t>
+    <t>efbc:TermCode[@listName='contract-detail']/text()='publ-ser-obl'</t>
   </si>
   <si>
     <t>?this epo:hasPublicServiceObligationsDescription ?value .</t>
   </si>
   <si>
-    <t>cbc:TermCode[@listName='contract-detail']/text()='soc-stand'</t>
+    <t>efbc:TermCode[@listName='contract-detail']/text()='soc-stand'</t>
   </si>
   <si>
     <t>?this epo:hasSocialStandardsDescription ?value .</t>

</xml_diff>